<commit_message>
update VRP network generation and BPR data files
</commit_message>
<xml_diff>
--- a/path_schedule_result.xlsx
+++ b/path_schedule_result.xlsx
@@ -492,13 +492,13 @@
         <v>9</v>
       </c>
       <c r="C3" t="n">
-        <v>471</v>
+        <v>473.7</v>
       </c>
       <c r="D3" t="n">
         <v>108.96</v>
       </c>
       <c r="E3" t="n">
-        <v>96.3</v>
+        <v>125.4</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -514,13 +514,13 @@
         <v>10</v>
       </c>
       <c r="C4" t="n">
-        <v>472.2</v>
+        <v>482.1</v>
       </c>
       <c r="D4" t="n">
         <v>80.59999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>146.9</v>
+        <v>155.7</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -602,17 +602,17 @@
         <v>4</v>
       </c>
       <c r="C8" t="n">
-        <v>235.2</v>
+        <v>265.5</v>
       </c>
       <c r="D8" t="n">
-        <v>40.29</v>
+        <v>68.06999999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>46.9</v>
+        <v>80.7</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Customer_30 → Customer_58 → Customer_37 → Customer_3</t>
+          <t>Customer_30 → Customer_58 → Customer_62 → Customer_47</t>
         </is>
       </c>
     </row>
@@ -674,11 +674,11 @@
         <v>36.72</v>
       </c>
       <c r="E11" t="n">
-        <v>75.5</v>
+        <v>75.8</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Customer_57 → Customer_47 → Customer_63</t>
+          <t>Customer_57 → Customer_3 → Customer_63</t>
         </is>
       </c>
     </row>
@@ -687,20 +687,20 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C12" t="n">
-        <v>248.9</v>
+        <v>460.6</v>
       </c>
       <c r="D12" t="n">
-        <v>59.8</v>
+        <v>129.92</v>
       </c>
       <c r="E12" t="n">
-        <v>112.5</v>
+        <v>149</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Customer_73 → Customer_79 → Customer_7 → Customer_78</t>
+          <t>Customer_73 → Customer_79 → Customer_37 → Customer_78 → Customer_43 → Customer_76 → Customer_11 → Customer_45</t>
         </is>
       </c>
     </row>
@@ -709,20 +709,20 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C13" t="n">
-        <v>204.8</v>
+        <v>159.8</v>
       </c>
       <c r="D13" t="n">
         <v>32.25</v>
       </c>
       <c r="E13" t="n">
-        <v>47.6</v>
+        <v>46.7</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Customer_21 → Customer_4 → Customer_45 → Customer_36</t>
+          <t>Customer_21 → Customer_4 → Customer_36</t>
         </is>
       </c>
     </row>
@@ -731,20 +731,20 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C14" t="n">
-        <v>202.1</v>
+        <v>105.8</v>
       </c>
       <c r="D14" t="n">
-        <v>42.3</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Customer_66 → Customer_62 → Customer_11 → Customer_76</t>
+          <t>Customer_66 → Customer_56</t>
         </is>
       </c>
     </row>
@@ -756,17 +756,17 @@
         <v>2</v>
       </c>
       <c r="C15" t="n">
-        <v>102</v>
+        <v>130.6</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>19.53</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Customer_20 → Customer_53</t>
+          <t>Customer_7 → Customer_20</t>
         </is>
       </c>
     </row>
@@ -775,20 +775,20 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>99</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="D16" t="n">
-        <v>7.82</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Customer_43 → Customer_8</t>
+          <t>Customer_5</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
         <v>1</v>
       </c>
       <c r="C17" t="n">
-        <v>67.09999999999999</v>
+        <v>54.9</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -810,7 +810,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Customer_5</t>
+          <t>Customer_29</t>
         </is>
       </c>
     </row>
@@ -819,20 +819,20 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" t="n">
-        <v>54.9</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>11.52</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Customer_29</t>
+          <t>Customer_53 → Customer_24</t>
         </is>
       </c>
     </row>
@@ -841,20 +841,20 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19" t="n">
-        <v>131.3</v>
+        <v>51.9</v>
       </c>
       <c r="D19" t="n">
-        <v>26.61</v>
+        <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>77.90000000000001</v>
+        <v>0</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Customer_56 → Customer_17</t>
+          <t>Customer_8</t>
         </is>
       </c>
     </row>
@@ -910,17 +910,17 @@
         <v>2</v>
       </c>
       <c r="C22" t="n">
-        <v>120.9</v>
+        <v>116.7</v>
       </c>
       <c r="D22" t="n">
-        <v>24.59</v>
+        <v>15.02</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Customer_24 → Customer_10</t>
+          <t>Customer_10 → Customer_42</t>
         </is>
       </c>
     </row>
@@ -954,7 +954,7 @@
         <v>1</v>
       </c>
       <c r="C24" t="n">
-        <v>52.7</v>
+        <v>64.8</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -964,7 +964,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Customer_42</t>
+          <t>Customer_19</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
         <v>1</v>
       </c>
       <c r="C25" t="n">
-        <v>64.8</v>
+        <v>34.3</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -986,7 +986,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Customer_19</t>
+          <t>Customer_17</t>
         </is>
       </c>
     </row>
@@ -1558,16 +1558,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3418</v>
+        <v>3420</v>
       </c>
       <c r="E10" t="n">
-        <v>112.3</v>
+        <v>115.2</v>
       </c>
       <c r="F10" t="n">
-        <v>142.3</v>
+        <v>145.2</v>
       </c>
       <c r="G10" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H10" t="n">
         <v>5.6</v>
@@ -1590,7 +1590,7 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>8.300000000000001</v>
+        <v>12.8</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1614,10 +1614,10 @@
         <v>2805</v>
       </c>
       <c r="E11" t="n">
-        <v>151.1</v>
+        <v>154.1</v>
       </c>
       <c r="F11" t="n">
-        <v>196.1</v>
+        <v>199.1</v>
       </c>
       <c r="G11" t="n">
         <v>8.9</v>
@@ -1667,10 +1667,10 @@
         <v>3909</v>
       </c>
       <c r="E12" t="n">
-        <v>206.5</v>
+        <v>209.4</v>
       </c>
       <c r="F12" t="n">
-        <v>251.5</v>
+        <v>254.4</v>
       </c>
       <c r="G12" t="n">
         <v>10.3</v>
@@ -1720,10 +1720,10 @@
         <v>6402</v>
       </c>
       <c r="E13" t="n">
-        <v>262.9</v>
+        <v>265.8</v>
       </c>
       <c r="F13" t="n">
-        <v>292.9</v>
+        <v>295.8</v>
       </c>
       <c r="G13" t="n">
         <v>11.4</v>
@@ -1773,10 +1773,10 @@
         <v>4632</v>
       </c>
       <c r="E14" t="n">
-        <v>306.1</v>
+        <v>309</v>
       </c>
       <c r="F14" t="n">
-        <v>351.1</v>
+        <v>354</v>
       </c>
       <c r="G14" t="n">
         <v>13.2</v>
@@ -1826,10 +1826,10 @@
         <v>8690</v>
       </c>
       <c r="E15" t="n">
-        <v>379.3</v>
+        <v>382.3</v>
       </c>
       <c r="F15" t="n">
-        <v>409.3</v>
+        <v>412.3</v>
       </c>
       <c r="G15" t="n">
         <v>28.3</v>
@@ -1876,16 +1876,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>9442</v>
+        <v>9443</v>
       </c>
       <c r="E16" t="n">
-        <v>441</v>
+        <v>443.7</v>
       </c>
       <c r="F16" t="n">
-        <v>471</v>
+        <v>473.7</v>
       </c>
       <c r="G16" t="n">
-        <v>31.7</v>
+        <v>31.4</v>
       </c>
       <c r="H16" t="n">
         <v>28.16</v>
@@ -1897,20 +1897,24 @@
         <v>11.392</v>
       </c>
       <c r="K16" t="n">
-        <v>257.9</v>
+        <v>282</v>
       </c>
       <c r="L16" t="n">
-        <v>257.9</v>
+        <v>282</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" t="inlineStr"/>
+        <v>24.7</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2082,16 +2086,16 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>3769</v>
+        <v>3771</v>
       </c>
       <c r="E20" t="n">
-        <v>182.5</v>
+        <v>185.1</v>
       </c>
       <c r="F20" t="n">
-        <v>212.5</v>
+        <v>215.1</v>
       </c>
       <c r="G20" t="n">
-        <v>2.4</v>
+        <v>5</v>
       </c>
       <c r="H20" t="n">
         <v>1.57</v>
@@ -2114,7 +2118,7 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>2.2</v>
+        <v>4.7</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2135,16 +2139,16 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1993</v>
+        <v>1995</v>
       </c>
       <c r="E21" t="n">
-        <v>214.4</v>
+        <v>220.6</v>
       </c>
       <c r="F21" t="n">
-        <v>259.4</v>
+        <v>265.6</v>
       </c>
       <c r="G21" t="n">
-        <v>1.9</v>
+        <v>5.5</v>
       </c>
       <c r="H21" t="n">
         <v>1.24</v>
@@ -2156,20 +2160,24 @@
         <v>32.035</v>
       </c>
       <c r="K21" t="n">
-        <v>280.4</v>
+        <v>282</v>
       </c>
       <c r="L21" t="n">
-        <v>280.4</v>
+        <v>282</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" t="inlineStr"/>
+        <v>4.8</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2184,16 +2192,16 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>836</v>
+        <v>838</v>
       </c>
       <c r="E22" t="n">
-        <v>261.2</v>
+        <v>271</v>
       </c>
       <c r="F22" t="n">
-        <v>291.2</v>
+        <v>301</v>
       </c>
       <c r="G22" t="n">
-        <v>1.9</v>
+        <v>5.5</v>
       </c>
       <c r="H22" t="n">
         <v>1.24</v>
@@ -2205,20 +2213,24 @@
         <v>26.506</v>
       </c>
       <c r="K22" t="n">
-        <v>278.8</v>
+        <v>282</v>
       </c>
       <c r="L22" t="n">
-        <v>278.8</v>
+        <v>282</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N22" t="n">
-        <v>0</v>
-      </c>
-      <c r="O22" t="inlineStr"/>
+        <v>4.5</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2236,10 +2248,10 @@
         <v>2351</v>
       </c>
       <c r="E23" t="n">
-        <v>297.4</v>
+        <v>307.2</v>
       </c>
       <c r="F23" t="n">
-        <v>327.4</v>
+        <v>337.2</v>
       </c>
       <c r="G23" t="n">
         <v>6.1</v>
@@ -2265,7 +2277,7 @@
         </is>
       </c>
       <c r="N23" t="n">
-        <v>8.800000000000001</v>
+        <v>5.7</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2286,16 +2298,16 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>3095</v>
+        <v>3096</v>
       </c>
       <c r="E24" t="n">
-        <v>334.5</v>
+        <v>344.4</v>
       </c>
       <c r="F24" t="n">
-        <v>364.5</v>
+        <v>374.4</v>
       </c>
       <c r="G24" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="H24" t="n">
         <v>6.5</v>
@@ -2307,24 +2319,20 @@
         <v>20.899</v>
       </c>
       <c r="K24" t="n">
-        <v>282</v>
+        <v>275</v>
       </c>
       <c r="L24" t="n">
-        <v>282</v>
+        <v>275</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N24" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2342,10 +2350,10 @@
         <v>5048</v>
       </c>
       <c r="E25" t="n">
-        <v>382.3</v>
+        <v>392.2</v>
       </c>
       <c r="F25" t="n">
-        <v>412.3</v>
+        <v>422.2</v>
       </c>
       <c r="G25" t="n">
         <v>17.8</v>
@@ -2371,7 +2379,7 @@
         </is>
       </c>
       <c r="N25" t="n">
-        <v>16.5</v>
+        <v>23.4</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2395,13 +2403,13 @@
         <v>5324</v>
       </c>
       <c r="E26" t="n">
-        <v>442.2</v>
+        <v>452.1</v>
       </c>
       <c r="F26" t="n">
-        <v>472.2</v>
+        <v>482.1</v>
       </c>
       <c r="G26" t="n">
-        <v>29.9</v>
+        <v>29.8</v>
       </c>
       <c r="H26" t="n">
         <v>26.61</v>
@@ -3034,7 +3042,7 @@
         <v>34.69</v>
       </c>
       <c r="J38" t="n">
-        <v>49.915</v>
+        <v>49.679</v>
       </c>
       <c r="K38" t="n">
         <v>268.3</v>
@@ -3083,7 +3091,7 @@
         <v>1.946</v>
       </c>
       <c r="J39" t="n">
-        <v>15.225</v>
+        <v>14.989</v>
       </c>
       <c r="K39" t="n">
         <v>282</v>
@@ -3097,7 +3105,7 @@
         </is>
       </c>
       <c r="N39" t="n">
-        <v>29.7</v>
+        <v>29.6</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
@@ -3114,29 +3122,29 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Customer_37</t>
+          <t>Customer_62</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>9338</v>
+        <v>9366</v>
       </c>
       <c r="E40" t="n">
-        <v>132.9</v>
+        <v>142</v>
       </c>
       <c r="F40" t="n">
-        <v>177.9</v>
+        <v>187</v>
       </c>
       <c r="G40" t="n">
-        <v>20.8</v>
+        <v>29.9</v>
       </c>
       <c r="H40" t="n">
-        <v>19.05</v>
+        <v>27.36</v>
       </c>
       <c r="I40" t="n">
-        <v>1.776</v>
+        <v>1.879</v>
       </c>
       <c r="J40" t="n">
-        <v>13.279</v>
+        <v>13.043</v>
       </c>
       <c r="K40" t="n">
         <v>282</v>
@@ -3150,11 +3158,11 @@
         </is>
       </c>
       <c r="N40" t="n">
-        <v>17.2</v>
+        <v>24.6</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>14</t>
         </is>
       </c>
     </row>
@@ -3167,45 +3175,49 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Customer_3</t>
+          <t>Customer_47</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>2134</v>
+        <v>9810</v>
       </c>
       <c r="E41" t="n">
-        <v>190.2</v>
+        <v>220.5</v>
       </c>
       <c r="F41" t="n">
-        <v>235.2</v>
+        <v>265.5</v>
       </c>
       <c r="G41" t="n">
-        <v>12.2</v>
+        <v>33.5</v>
       </c>
       <c r="H41" t="n">
-        <v>11.23</v>
+        <v>30.69</v>
       </c>
       <c r="I41" t="n">
-        <v>1.503</v>
+        <v>1.164</v>
       </c>
       <c r="J41" t="n">
-        <v>11.503</v>
+        <v>11.164</v>
       </c>
       <c r="K41" t="n">
-        <v>272.3</v>
+        <v>282</v>
       </c>
       <c r="L41" t="n">
-        <v>272.3</v>
+        <v>282</v>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N41" t="n">
-        <v>0</v>
-      </c>
-      <c r="O41" t="inlineStr"/>
+        <v>26.4</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -3656,13 +3668,13 @@
         <v>29.692</v>
       </c>
       <c r="J50" t="n">
-        <v>49.293</v>
+        <v>49.632</v>
       </c>
       <c r="K50" t="n">
-        <v>255</v>
+        <v>254.9</v>
       </c>
       <c r="L50" t="n">
-        <v>255</v>
+        <v>254.9</v>
       </c>
       <c r="M50" t="inlineStr">
         <is>
@@ -3683,11 +3695,11 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Customer_47</t>
+          <t>Customer_3</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>3272</v>
+        <v>3266</v>
       </c>
       <c r="E51" t="n">
         <v>68.90000000000001</v>
@@ -3702,10 +3714,10 @@
         <v>18.62</v>
       </c>
       <c r="I51" t="n">
-        <v>1.164</v>
+        <v>1.503</v>
       </c>
       <c r="J51" t="n">
-        <v>19.601</v>
+        <v>19.94</v>
       </c>
       <c r="K51" t="n">
         <v>282</v>
@@ -3719,7 +3731,7 @@
         </is>
       </c>
       <c r="N51" t="n">
-        <v>56.6</v>
+        <v>56.8</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
@@ -3740,7 +3752,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>8272</v>
+        <v>6742</v>
       </c>
       <c r="E52" t="n">
         <v>134.9</v>
@@ -3772,7 +3784,7 @@
         </is>
       </c>
       <c r="N52" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
@@ -3813,13 +3825,13 @@
         <v>4.608</v>
       </c>
       <c r="J53" t="n">
-        <v>49.028</v>
+        <v>46.94</v>
       </c>
       <c r="K53" t="n">
-        <v>254.9</v>
+        <v>255.7</v>
       </c>
       <c r="L53" t="n">
-        <v>254.9</v>
+        <v>255.7</v>
       </c>
       <c r="M53" t="inlineStr">
         <is>
@@ -3862,7 +3874,7 @@
         <v>10.495</v>
       </c>
       <c r="J54" t="n">
-        <v>44.42</v>
+        <v>42.332</v>
       </c>
       <c r="K54" t="n">
         <v>282</v>
@@ -3876,7 +3888,7 @@
         </is>
       </c>
       <c r="N54" t="n">
-        <v>51.5</v>
+        <v>50.2</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
@@ -3893,29 +3905,29 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Customer_7</t>
+          <t>Customer_37</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>11487</v>
+        <v>11447</v>
       </c>
       <c r="E55" t="n">
-        <v>133.2</v>
+        <v>131.2</v>
       </c>
       <c r="F55" t="n">
-        <v>178.2</v>
+        <v>176.2</v>
       </c>
       <c r="G55" t="n">
-        <v>22.6</v>
+        <v>20.7</v>
       </c>
       <c r="H55" t="n">
-        <v>20.74</v>
+        <v>18.96</v>
       </c>
       <c r="I55" t="n">
-        <v>14.668</v>
+        <v>1.776</v>
       </c>
       <c r="J55" t="n">
-        <v>33.925</v>
+        <v>31.837</v>
       </c>
       <c r="K55" t="n">
         <v>282</v>
@@ -3929,7 +3941,7 @@
         </is>
       </c>
       <c r="N55" t="n">
-        <v>30.9</v>
+        <v>27.4</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
@@ -3950,25 +3962,25 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>411</v>
+        <v>7397</v>
       </c>
       <c r="E56" t="n">
-        <v>203.9</v>
+        <v>200</v>
       </c>
       <c r="F56" t="n">
-        <v>248.9</v>
+        <v>245</v>
       </c>
       <c r="G56" t="n">
-        <v>25.7</v>
+        <v>23.8</v>
       </c>
       <c r="H56" t="n">
-        <v>23.58</v>
+        <v>21.79</v>
       </c>
       <c r="I56" t="n">
         <v>9.257</v>
       </c>
       <c r="J56" t="n">
-        <v>19.257</v>
+        <v>30.061</v>
       </c>
       <c r="K56" t="n">
         <v>282</v>
@@ -3982,7 +3994,7 @@
         </is>
       </c>
       <c r="N56" t="n">
-        <v>30.1</v>
+        <v>27</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
@@ -3992,87 +4004,89 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B57" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Customer_21</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>VIR</t>
-        </is>
+          <t>Customer_43</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>11374</v>
       </c>
       <c r="E57" t="n">
-        <v>4.6</v>
+        <v>285.4</v>
       </c>
       <c r="F57" t="n">
-        <v>49.6</v>
+        <v>315.4</v>
       </c>
       <c r="G57" t="n">
-        <v>0</v>
+        <v>40.4</v>
       </c>
       <c r="H57" t="n">
-        <v>0</v>
+        <v>37.02</v>
       </c>
       <c r="I57" t="n">
-        <v>26.403</v>
+        <v>5.942</v>
       </c>
       <c r="J57" t="n">
-        <v>48.883</v>
+        <v>20.804</v>
       </c>
       <c r="K57" t="n">
-        <v>275.3</v>
+        <v>282</v>
       </c>
       <c r="L57" t="n">
-        <v>275.3</v>
+        <v>282</v>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N57" t="n">
-        <v>0</v>
-      </c>
-      <c r="O57" t="inlineStr"/>
+        <v>44.5</v>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B58" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Customer_4</t>
+          <t>Customer_76</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>5828</v>
+        <v>2431</v>
       </c>
       <c r="E58" t="n">
-        <v>77.90000000000001</v>
+        <v>315.4</v>
       </c>
       <c r="F58" t="n">
-        <v>107.9</v>
+        <v>345.4</v>
       </c>
       <c r="G58" t="n">
-        <v>28.2</v>
+        <v>0</v>
       </c>
       <c r="H58" t="n">
-        <v>25.89</v>
+        <v>0</v>
       </c>
       <c r="I58" t="n">
-        <v>5.157</v>
+        <v>1.697</v>
       </c>
       <c r="J58" t="n">
-        <v>22.48</v>
+        <v>14.862</v>
       </c>
       <c r="K58" t="n">
         <v>282</v>
@@ -4082,56 +4096,52 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N58" t="n">
-        <v>47.6</v>
-      </c>
-      <c r="O58" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B59" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Customer_45</t>
+          <t>Customer_11</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>180</v>
+        <v>4286</v>
       </c>
       <c r="E59" t="n">
-        <v>107.9</v>
+        <v>348.8</v>
       </c>
       <c r="F59" t="n">
-        <v>152.9</v>
+        <v>378.8</v>
       </c>
       <c r="G59" t="n">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="H59" t="n">
-        <v>0</v>
+        <v>3.12</v>
       </c>
       <c r="I59" t="n">
-        <v>1.469</v>
+        <v>1.696</v>
       </c>
       <c r="J59" t="n">
-        <v>17.323</v>
+        <v>13.165</v>
       </c>
       <c r="K59" t="n">
-        <v>282</v>
+        <v>279.2</v>
       </c>
       <c r="L59" t="n">
-        <v>282</v>
+        <v>279.2</v>
       </c>
       <c r="M59" t="inlineStr">
         <is>
@@ -4145,42 +4155,42 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B60" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Customer_36</t>
+          <t>Customer_45</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>2524</v>
+        <v>4815</v>
       </c>
       <c r="E60" t="n">
-        <v>159.8</v>
+        <v>415.6</v>
       </c>
       <c r="F60" t="n">
-        <v>204.8</v>
+        <v>460.6</v>
       </c>
       <c r="G60" t="n">
-        <v>6.9</v>
+        <v>36.8</v>
       </c>
       <c r="H60" t="n">
-        <v>6.36</v>
+        <v>33.55</v>
       </c>
       <c r="I60" t="n">
-        <v>5.854</v>
+        <v>1.469</v>
       </c>
       <c r="J60" t="n">
-        <v>15.854</v>
+        <v>11.469</v>
       </c>
       <c r="K60" t="n">
-        <v>276</v>
+        <v>250.1</v>
       </c>
       <c r="L60" t="n">
-        <v>276</v>
+        <v>250.1</v>
       </c>
       <c r="M60" t="inlineStr">
         <is>
@@ -4194,14 +4204,14 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B61" t="n">
         <v>1</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Customer_66</t>
+          <t>Customer_21</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -4210,10 +4220,10 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>20.8</v>
+        <v>4.6</v>
       </c>
       <c r="F61" t="n">
-        <v>50.8</v>
+        <v>49.6</v>
       </c>
       <c r="G61" t="n">
         <v>0</v>
@@ -4222,16 +4232,16 @@
         <v>0</v>
       </c>
       <c r="I61" t="n">
-        <v>30.607</v>
+        <v>26.403</v>
       </c>
       <c r="J61" t="n">
-        <v>45.879</v>
+        <v>47.414</v>
       </c>
       <c r="K61" t="n">
-        <v>253.1</v>
+        <v>275.4</v>
       </c>
       <c r="L61" t="n">
-        <v>253.1</v>
+        <v>275.4</v>
       </c>
       <c r="M61" t="inlineStr">
         <is>
@@ -4245,91 +4255,95 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B62" t="n">
         <v>2</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Customer_62</t>
+          <t>Customer_4</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>3763</v>
+        <v>5828</v>
       </c>
       <c r="E62" t="n">
-        <v>60.7</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="F62" t="n">
-        <v>105.7</v>
+        <v>107.9</v>
       </c>
       <c r="G62" t="n">
-        <v>9.9</v>
+        <v>28.2</v>
       </c>
       <c r="H62" t="n">
-        <v>9.06</v>
+        <v>25.89</v>
       </c>
       <c r="I62" t="n">
-        <v>1.879</v>
+        <v>5.157</v>
       </c>
       <c r="J62" t="n">
-        <v>15.272</v>
+        <v>21.011</v>
       </c>
       <c r="K62" t="n">
-        <v>239.3</v>
+        <v>282</v>
       </c>
       <c r="L62" t="n">
-        <v>239.3</v>
+        <v>282</v>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N62" t="n">
-        <v>0</v>
-      </c>
-      <c r="O62" t="inlineStr"/>
+        <v>46.7</v>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B63" t="n">
         <v>3</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Customer_11</t>
+          <t>Customer_36</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>9774</v>
+        <v>181</v>
       </c>
       <c r="E63" t="n">
-        <v>138.7</v>
+        <v>114.8</v>
       </c>
       <c r="F63" t="n">
-        <v>168.7</v>
+        <v>159.8</v>
       </c>
       <c r="G63" t="n">
-        <v>33</v>
+        <v>6.9</v>
       </c>
       <c r="H63" t="n">
-        <v>30.11</v>
+        <v>6.36</v>
       </c>
       <c r="I63" t="n">
-        <v>1.696</v>
+        <v>5.854</v>
       </c>
       <c r="J63" t="n">
-        <v>13.393</v>
+        <v>15.854</v>
       </c>
       <c r="K63" t="n">
-        <v>211.9</v>
+        <v>275.5</v>
       </c>
       <c r="L63" t="n">
-        <v>211.9</v>
+        <v>275.5</v>
       </c>
       <c r="M63" t="inlineStr">
         <is>
@@ -4346,39 +4360,41 @@
         <v>12</v>
       </c>
       <c r="B64" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Customer_76</t>
-        </is>
-      </c>
-      <c r="D64" t="n">
-        <v>606</v>
+          <t>Customer_66</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
       </c>
       <c r="E64" t="n">
-        <v>172.1</v>
+        <v>20.8</v>
       </c>
       <c r="F64" t="n">
-        <v>202.1</v>
+        <v>50.8</v>
       </c>
       <c r="G64" t="n">
-        <v>3.4</v>
+        <v>0</v>
       </c>
       <c r="H64" t="n">
-        <v>3.12</v>
+        <v>0</v>
       </c>
       <c r="I64" t="n">
-        <v>1.697</v>
+        <v>30.607</v>
       </c>
       <c r="J64" t="n">
-        <v>11.697</v>
+        <v>49.861</v>
       </c>
       <c r="K64" t="n">
-        <v>209.2</v>
+        <v>251.6</v>
       </c>
       <c r="L64" t="n">
-        <v>209.2</v>
+        <v>251.6</v>
       </c>
       <c r="M64" t="inlineStr">
         <is>
@@ -4392,44 +4408,42 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Customer_20</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>VIR</t>
-        </is>
+          <t>Customer_56</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>3735</v>
       </c>
       <c r="E65" t="n">
-        <v>27</v>
+        <v>60.8</v>
       </c>
       <c r="F65" t="n">
-        <v>72</v>
+        <v>105.8</v>
       </c>
       <c r="G65" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H65" t="n">
-        <v>0</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="I65" t="n">
-        <v>23.057</v>
+        <v>9.254</v>
       </c>
       <c r="J65" t="n">
-        <v>44.795</v>
+        <v>19.254</v>
       </c>
       <c r="K65" t="n">
-        <v>245</v>
+        <v>237.1</v>
       </c>
       <c r="L65" t="n">
-        <v>245</v>
+        <v>237.1</v>
       </c>
       <c r="M65" t="inlineStr">
         <is>
@@ -4446,21 +4460,23 @@
         <v>13</v>
       </c>
       <c r="B66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Customer_53</t>
-        </is>
-      </c>
-      <c r="D66" t="n">
-        <v>1119</v>
+          <t>Customer_7</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
       </c>
       <c r="E66" t="n">
-        <v>72</v>
+        <v>19.3</v>
       </c>
       <c r="F66" t="n">
-        <v>102</v>
+        <v>64.3</v>
       </c>
       <c r="G66" t="n">
         <v>0</v>
@@ -4469,16 +4485,16 @@
         <v>0</v>
       </c>
       <c r="I66" t="n">
-        <v>11.738</v>
+        <v>14.668</v>
       </c>
       <c r="J66" t="n">
-        <v>21.738</v>
+        <v>47.725</v>
       </c>
       <c r="K66" t="n">
-        <v>245</v>
+        <v>254.5</v>
       </c>
       <c r="L66" t="n">
-        <v>245</v>
+        <v>254.5</v>
       </c>
       <c r="M66" t="inlineStr">
         <is>
@@ -4492,44 +4508,42 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Customer_43</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>VIR</t>
-        </is>
+          <t>Customer_20</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>10581</v>
       </c>
       <c r="E67" t="n">
-        <v>30.5</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="F67" t="n">
-        <v>60.5</v>
+        <v>130.6</v>
       </c>
       <c r="G67" t="n">
-        <v>0</v>
+        <v>21.3</v>
       </c>
       <c r="H67" t="n">
-        <v>0</v>
+        <v>19.53</v>
       </c>
       <c r="I67" t="n">
-        <v>5.942</v>
+        <v>23.057</v>
       </c>
       <c r="J67" t="n">
-        <v>47.492</v>
+        <v>33.057</v>
       </c>
       <c r="K67" t="n">
-        <v>238.9</v>
+        <v>224.1</v>
       </c>
       <c r="L67" t="n">
-        <v>238.9</v>
+        <v>224.1</v>
       </c>
       <c r="M67" t="inlineStr">
         <is>
@@ -4546,39 +4560,41 @@
         <v>14</v>
       </c>
       <c r="B68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Customer_8</t>
-        </is>
-      </c>
-      <c r="D68" t="n">
-        <v>2447</v>
+          <t>Customer_5</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
       </c>
       <c r="E68" t="n">
-        <v>69</v>
+        <v>22.1</v>
       </c>
       <c r="F68" t="n">
-        <v>99</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="G68" t="n">
-        <v>8.5</v>
+        <v>0</v>
       </c>
       <c r="H68" t="n">
-        <v>7.82</v>
+        <v>0</v>
       </c>
       <c r="I68" t="n">
-        <v>31.55</v>
+        <v>35.722</v>
       </c>
       <c r="J68" t="n">
-        <v>41.55</v>
+        <v>45.722</v>
       </c>
       <c r="K68" t="n">
-        <v>226.8</v>
+        <v>252</v>
       </c>
       <c r="L68" t="n">
-        <v>226.8</v>
+        <v>252</v>
       </c>
       <c r="M68" t="inlineStr">
         <is>
@@ -4599,7 +4615,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Customer_5</t>
+          <t>Customer_29</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -4608,10 +4624,10 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>22.1</v>
+        <v>9.9</v>
       </c>
       <c r="F69" t="n">
-        <v>67.09999999999999</v>
+        <v>54.9</v>
       </c>
       <c r="G69" t="n">
         <v>0</v>
@@ -4620,16 +4636,16 @@
         <v>0</v>
       </c>
       <c r="I69" t="n">
-        <v>35.722</v>
+        <v>32.083</v>
       </c>
       <c r="J69" t="n">
-        <v>45.722</v>
+        <v>42.083</v>
       </c>
       <c r="K69" t="n">
-        <v>252</v>
+        <v>270.2</v>
       </c>
       <c r="L69" t="n">
-        <v>252</v>
+        <v>270.2</v>
       </c>
       <c r="M69" t="inlineStr">
         <is>
@@ -4650,7 +4666,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Customer_29</t>
+          <t>Customer_53</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -4659,10 +4675,10 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>9.9</v>
+        <v>27</v>
       </c>
       <c r="F70" t="n">
-        <v>54.9</v>
+        <v>57</v>
       </c>
       <c r="G70" t="n">
         <v>0</v>
@@ -4671,16 +4687,16 @@
         <v>0</v>
       </c>
       <c r="I70" t="n">
-        <v>32.083</v>
+        <v>11.738</v>
       </c>
       <c r="J70" t="n">
-        <v>42.083</v>
+        <v>47.2</v>
       </c>
       <c r="K70" t="n">
-        <v>270.2</v>
+        <v>243.9</v>
       </c>
       <c r="L70" t="n">
-        <v>270.2</v>
+        <v>243.9</v>
       </c>
       <c r="M70" t="inlineStr">
         <is>
@@ -4694,44 +4710,42 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Customer_56</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>VIR</t>
-        </is>
+          <t>Customer_24</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>3031</v>
       </c>
       <c r="E71" t="n">
-        <v>26.4</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="F71" t="n">
-        <v>71.40000000000001</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="G71" t="n">
-        <v>0</v>
+        <v>12.6</v>
       </c>
       <c r="H71" t="n">
-        <v>0</v>
+        <v>11.52</v>
       </c>
       <c r="I71" t="n">
-        <v>9.254</v>
+        <v>25.462</v>
       </c>
       <c r="J71" t="n">
-        <v>46.578</v>
+        <v>35.462</v>
       </c>
       <c r="K71" t="n">
-        <v>246</v>
+        <v>226.1</v>
       </c>
       <c r="L71" t="n">
-        <v>246</v>
+        <v>226.1</v>
       </c>
       <c r="M71" t="inlineStr">
         <is>
@@ -4748,53 +4762,51 @@
         <v>17</v>
       </c>
       <c r="B72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Customer_17</t>
-        </is>
-      </c>
-      <c r="D72" t="n">
-        <v>9128</v>
+          <t>Customer_8</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
       </c>
       <c r="E72" t="n">
-        <v>101.3</v>
+        <v>21.9</v>
       </c>
       <c r="F72" t="n">
-        <v>131.3</v>
+        <v>51.9</v>
       </c>
       <c r="G72" t="n">
-        <v>29.8</v>
+        <v>0</v>
       </c>
       <c r="H72" t="n">
-        <v>26.61</v>
+        <v>0</v>
       </c>
       <c r="I72" t="n">
-        <v>27.324</v>
+        <v>31.55</v>
       </c>
       <c r="J72" t="n">
-        <v>37.324</v>
+        <v>41.55</v>
       </c>
       <c r="K72" t="n">
-        <v>282</v>
+        <v>253.4</v>
       </c>
       <c r="L72" t="n">
-        <v>282</v>
+        <v>253.4</v>
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N72" t="n">
-        <v>77.90000000000001</v>
-      </c>
-      <c r="O72" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -4907,7 +4919,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Customer_24</t>
+          <t>Customer_10</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -4916,10 +4928,10 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>18.6</v>
+        <v>9.5</v>
       </c>
       <c r="F75" t="n">
-        <v>48.6</v>
+        <v>54.5</v>
       </c>
       <c r="G75" t="n">
         <v>0</v>
@@ -4928,16 +4940,16 @@
         <v>0</v>
       </c>
       <c r="I75" t="n">
-        <v>25.462</v>
+        <v>14.093</v>
       </c>
       <c r="J75" t="n">
-        <v>49.555</v>
+        <v>48.517</v>
       </c>
       <c r="K75" t="n">
-        <v>255.5</v>
+        <v>268.3</v>
       </c>
       <c r="L75" t="n">
-        <v>255.5</v>
+        <v>268.3</v>
       </c>
       <c r="M75" t="inlineStr">
         <is>
@@ -4958,35 +4970,35 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Customer_10</t>
+          <t>Customer_42</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>6093</v>
+        <v>598</v>
       </c>
       <c r="E76" t="n">
-        <v>75.90000000000001</v>
+        <v>71.7</v>
       </c>
       <c r="F76" t="n">
-        <v>120.9</v>
+        <v>116.7</v>
       </c>
       <c r="G76" t="n">
-        <v>27.3</v>
+        <v>17.2</v>
       </c>
       <c r="H76" t="n">
-        <v>24.59</v>
+        <v>15.02</v>
       </c>
       <c r="I76" t="n">
-        <v>14.093</v>
+        <v>24.424</v>
       </c>
       <c r="J76" t="n">
-        <v>24.093</v>
+        <v>34.424</v>
       </c>
       <c r="K76" t="n">
-        <v>215.7</v>
+        <v>243.5</v>
       </c>
       <c r="L76" t="n">
-        <v>215.7</v>
+        <v>243.5</v>
       </c>
       <c r="M76" t="inlineStr">
         <is>
@@ -5058,7 +5070,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Customer_42</t>
+          <t>Customer_19</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -5067,10 +5079,10 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>7.7</v>
+        <v>19.8</v>
       </c>
       <c r="F78" t="n">
-        <v>52.7</v>
+        <v>64.8</v>
       </c>
       <c r="G78" t="n">
         <v>0</v>
@@ -5079,16 +5091,16 @@
         <v>0</v>
       </c>
       <c r="I78" t="n">
-        <v>24.424</v>
+        <v>16.088</v>
       </c>
       <c r="J78" t="n">
-        <v>34.424</v>
+        <v>26.088</v>
       </c>
       <c r="K78" t="n">
-        <v>273</v>
+        <v>261.6</v>
       </c>
       <c r="L78" t="n">
-        <v>273</v>
+        <v>261.6</v>
       </c>
       <c r="M78" t="inlineStr">
         <is>
@@ -5109,7 +5121,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Customer_19</t>
+          <t>Customer_17</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -5118,10 +5130,10 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>19.8</v>
+        <v>4.3</v>
       </c>
       <c r="F79" t="n">
-        <v>64.8</v>
+        <v>34.3</v>
       </c>
       <c r="G79" t="n">
         <v>0</v>
@@ -5130,16 +5142,16 @@
         <v>0</v>
       </c>
       <c r="I79" t="n">
-        <v>16.088</v>
+        <v>27.324</v>
       </c>
       <c r="J79" t="n">
-        <v>26.088</v>
+        <v>37.324</v>
       </c>
       <c r="K79" t="n">
-        <v>261.6</v>
+        <v>276.7</v>
       </c>
       <c r="L79" t="n">
-        <v>261.6</v>
+        <v>276.7</v>
       </c>
       <c r="M79" t="inlineStr">
         <is>
@@ -5264,7 +5276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5441,7 +5453,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>112.3</v>
+        <v>115.2</v>
       </c>
       <c r="D8" t="n">
         <v>282</v>
@@ -5450,7 +5462,7 @@
         <v>282</v>
       </c>
       <c r="F8" t="n">
-        <v>8.300000000000001</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="9">
@@ -5463,7 +5475,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>151.1</v>
+        <v>154.1</v>
       </c>
       <c r="D9" t="n">
         <v>282</v>
@@ -5485,7 +5497,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>206.5</v>
+        <v>209.4</v>
       </c>
       <c r="D10" t="n">
         <v>282</v>
@@ -5507,7 +5519,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>262.9</v>
+        <v>265.8</v>
       </c>
       <c r="D11" t="n">
         <v>282</v>
@@ -5529,7 +5541,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>306.1</v>
+        <v>309</v>
       </c>
       <c r="D12" t="n">
         <v>282</v>
@@ -5551,7 +5563,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>379.3</v>
+        <v>382.3</v>
       </c>
       <c r="D13" t="n">
         <v>282</v>
@@ -5565,15 +5577,15 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>90.2</v>
+        <v>443.7</v>
       </c>
       <c r="D14" t="n">
         <v>282</v>
@@ -5582,7 +5594,7 @@
         <v>282</v>
       </c>
       <c r="F14" t="n">
-        <v>87.40000000000001</v>
+        <v>24.7</v>
       </c>
     </row>
     <row r="15">
@@ -5595,7 +5607,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>135.2</v>
+        <v>90.2</v>
       </c>
       <c r="D15" t="n">
         <v>282</v>
@@ -5604,7 +5616,7 @@
         <v>282</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>87.40000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -5617,7 +5629,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>182.5</v>
+        <v>135.2</v>
       </c>
       <c r="D16" t="n">
         <v>282</v>
@@ -5626,7 +5638,7 @@
         <v>282</v>
       </c>
       <c r="F16" t="n">
-        <v>2.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -5639,7 +5651,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>297.4</v>
+        <v>185.1</v>
       </c>
       <c r="D17" t="n">
         <v>282</v>
@@ -5648,7 +5660,7 @@
         <v>282</v>
       </c>
       <c r="F17" t="n">
-        <v>8.800000000000001</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="18">
@@ -5661,7 +5673,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>334.5</v>
+        <v>220.6</v>
       </c>
       <c r="D18" t="n">
         <v>282</v>
@@ -5670,7 +5682,7 @@
         <v>282</v>
       </c>
       <c r="F18" t="n">
-        <v>6.8</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="19">
@@ -5679,11 +5691,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>31</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>382.3</v>
+        <v>271</v>
       </c>
       <c r="D19" t="n">
         <v>282</v>
@@ -5692,7 +5704,7 @@
         <v>282</v>
       </c>
       <c r="F19" t="n">
-        <v>16.5</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="20">
@@ -5701,11 +5713,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>31</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>442.2</v>
+        <v>307.2</v>
       </c>
       <c r="D20" t="n">
         <v>282</v>
@@ -5714,20 +5726,20 @@
         <v>282</v>
       </c>
       <c r="F20" t="n">
-        <v>25.2</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>61.4</v>
+        <v>392.2</v>
       </c>
       <c r="D21" t="n">
         <v>282</v>
@@ -5736,20 +5748,20 @@
         <v>282</v>
       </c>
       <c r="F21" t="n">
-        <v>24</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>109.8</v>
+        <v>452.1</v>
       </c>
       <c r="D22" t="n">
         <v>282</v>
@@ -5758,20 +5770,20 @@
         <v>282</v>
       </c>
       <c r="F22" t="n">
-        <v>3.9</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>28</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>92.8</v>
+        <v>61.4</v>
       </c>
       <c r="D23" t="n">
         <v>282</v>
@@ -5780,20 +5792,20 @@
         <v>282</v>
       </c>
       <c r="F23" t="n">
-        <v>69.7</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>28</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>126.3</v>
+        <v>109.8</v>
       </c>
       <c r="D24" t="n">
         <v>282</v>
@@ -5802,12 +5814,12 @@
         <v>282</v>
       </c>
       <c r="F24" t="n">
-        <v>3.2</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -5815,7 +5827,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>89.3</v>
+        <v>92.8</v>
       </c>
       <c r="D25" t="n">
         <v>282</v>
@@ -5824,12 +5836,12 @@
         <v>282</v>
       </c>
       <c r="F25" t="n">
-        <v>63</v>
+        <v>69.7</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -5837,7 +5849,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>145.9</v>
+        <v>126.3</v>
       </c>
       <c r="D26" t="n">
         <v>282</v>
@@ -5846,20 +5858,20 @@
         <v>282</v>
       </c>
       <c r="F26" t="n">
-        <v>28.2</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>67.09999999999999</v>
+        <v>89.3</v>
       </c>
       <c r="D27" t="n">
         <v>282</v>
@@ -5868,20 +5880,20 @@
         <v>282</v>
       </c>
       <c r="F27" t="n">
-        <v>29.7</v>
+        <v>63</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>132.9</v>
+        <v>145.9</v>
       </c>
       <c r="D28" t="n">
         <v>282</v>
@@ -5890,20 +5902,20 @@
         <v>282</v>
       </c>
       <c r="F28" t="n">
-        <v>17.2</v>
+        <v>28.2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>65.2</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="D29" t="n">
         <v>282</v>
@@ -5912,20 +5924,20 @@
         <v>282</v>
       </c>
       <c r="F29" t="n">
-        <v>29.2</v>
+        <v>29.6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>116</v>
+        <v>142</v>
       </c>
       <c r="D30" t="n">
         <v>282</v>
@@ -5934,20 +5946,20 @@
         <v>282</v>
       </c>
       <c r="F30" t="n">
-        <v>6</v>
+        <v>24.6</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>260.4</v>
+        <v>220.5</v>
       </c>
       <c r="D31" t="n">
         <v>282</v>
@@ -5956,20 +5968,20 @@
         <v>282</v>
       </c>
       <c r="F31" t="n">
-        <v>77</v>
+        <v>26.4</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>35</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>103.2</v>
+        <v>65.2</v>
       </c>
       <c r="D32" t="n">
         <v>282</v>
@@ -5978,12 +5990,12 @@
         <v>282</v>
       </c>
       <c r="F32" t="n">
-        <v>106</v>
+        <v>29.2</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -5991,7 +6003,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>164.1</v>
+        <v>116</v>
       </c>
       <c r="D33" t="n">
         <v>282</v>
@@ -6000,12 +6012,12 @@
         <v>282</v>
       </c>
       <c r="F33" t="n">
-        <v>13.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -6013,7 +6025,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>68.90000000000001</v>
+        <v>260.4</v>
       </c>
       <c r="D34" t="n">
         <v>282</v>
@@ -6022,20 +6034,20 @@
         <v>282</v>
       </c>
       <c r="F34" t="n">
-        <v>56.6</v>
+        <v>77</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>134.9</v>
+        <v>103.2</v>
       </c>
       <c r="D35" t="n">
         <v>282</v>
@@ -6044,20 +6056,20 @@
         <v>282</v>
       </c>
       <c r="F35" t="n">
-        <v>18.9</v>
+        <v>106</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>35</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>65.59999999999999</v>
+        <v>164.1</v>
       </c>
       <c r="D36" t="n">
         <v>282</v>
@@ -6066,12 +6078,12 @@
         <v>282</v>
       </c>
       <c r="F36" t="n">
-        <v>51.5</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -6079,7 +6091,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>133.2</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="D37" t="n">
         <v>282</v>
@@ -6088,20 +6100,20 @@
         <v>282</v>
       </c>
       <c r="F37" t="n">
-        <v>30.9</v>
+        <v>56.8</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>203.9</v>
+        <v>134.9</v>
       </c>
       <c r="D38" t="n">
         <v>282</v>
@@ -6110,12 +6122,12 @@
         <v>282</v>
       </c>
       <c r="F38" t="n">
-        <v>30.1</v>
+        <v>19</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -6123,7 +6135,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>77.90000000000001</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="D39" t="n">
         <v>282</v>
@@ -6132,20 +6144,20 @@
         <v>282</v>
       </c>
       <c r="F39" t="n">
-        <v>47.6</v>
+        <v>50.2</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>28</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>101.3</v>
+        <v>131.2</v>
       </c>
       <c r="D40" t="n">
         <v>282</v>
@@ -6154,7 +6166,73 @@
         <v>282</v>
       </c>
       <c r="F40" t="n">
+        <v>27.4</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>10</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>200</v>
+      </c>
+      <c r="D41" t="n">
+        <v>282</v>
+      </c>
+      <c r="E41" t="n">
+        <v>282</v>
+      </c>
+      <c r="F41" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>10</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>285.4</v>
+      </c>
+      <c r="D42" t="n">
+        <v>282</v>
+      </c>
+      <c r="E42" t="n">
+        <v>282</v>
+      </c>
+      <c r="F42" t="n">
+        <v>44.5</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>11</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
         <v>77.90000000000001</v>
+      </c>
+      <c r="D43" t="n">
+        <v>282</v>
+      </c>
+      <c r="E43" t="n">
+        <v>282</v>
+      </c>
+      <c r="F43" t="n">
+        <v>46.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update BRF model and scheduling results
</commit_message>
<xml_diff>
--- a/path_schedule_result.xlsx
+++ b/path_schedule_result.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,13 +470,13 @@
         <v>7</v>
       </c>
       <c r="C2" t="n">
-        <v>344</v>
+        <v>343.8</v>
       </c>
       <c r="D2" t="n">
         <v>62.61</v>
       </c>
       <c r="E2" t="n">
-        <v>62.2</v>
+        <v>89.8</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -533,20 +533,20 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C5" t="n">
-        <v>419.3</v>
+        <v>245.9</v>
       </c>
       <c r="D5" t="n">
-        <v>69.11</v>
+        <v>34.96</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>48.1</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Customer_46 → Customer_67 → Customer_35 → Customer_54 → Customer_41 → Customer_16 → Customer_9 → Customer_59 → Customer_62</t>
+          <t>Customer_46 → Customer_31 → Customer_67 → Customer_54 → Customer_18</t>
         </is>
       </c>
     </row>
@@ -555,20 +555,20 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C6" t="n">
-        <v>285.9</v>
+        <v>376</v>
       </c>
       <c r="D6" t="n">
-        <v>37.88</v>
+        <v>48.71</v>
       </c>
       <c r="E6" t="n">
-        <v>96.40000000000001</v>
+        <v>113.6</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Customer_72 → Customer_31 → Customer_15 → Customer_58 → Customer_27</t>
+          <t>Customer_72 → Customer_49 → Customer_27 → Customer_58 → Customer_74 → Customer_3 → Customer_15</t>
         </is>
       </c>
     </row>
@@ -577,20 +577,20 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>172.9</v>
+        <v>327.5</v>
       </c>
       <c r="D7" t="n">
-        <v>37.18</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="E7" t="n">
-        <v>90.59999999999999</v>
+        <v>140.6</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Customer_64 → Customer_48 → Customer_49</t>
+          <t>Customer_64 → Customer_35 → Customer_16 → Customer_41 → Customer_48 → Customer_59</t>
         </is>
       </c>
     </row>
@@ -621,20 +621,20 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>340.1</v>
+        <v>268.4</v>
       </c>
       <c r="D9" t="n">
-        <v>82.52</v>
+        <v>90.48999999999999</v>
       </c>
       <c r="E9" t="n">
-        <v>118.8</v>
+        <v>41.9</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Customer_18 → Customer_29 → Customer_3 → Customer_11 → Customer_74 → Customer_39</t>
+          <t>Customer_22 → Customer_7 → Customer_39 → Customer_61</t>
         </is>
       </c>
     </row>
@@ -646,17 +646,17 @@
         <v>4</v>
       </c>
       <c r="C10" t="n">
-        <v>233.4</v>
+        <v>257.9</v>
       </c>
       <c r="D10" t="n">
-        <v>44.7</v>
+        <v>70.48999999999999</v>
       </c>
       <c r="E10" t="n">
-        <v>41.9</v>
+        <v>0</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Customer_22 → Customer_7 → Customer_37 → Customer_61</t>
+          <t>Customer_25 → Customer_9 → Customer_62 → Customer_11</t>
         </is>
       </c>
     </row>
@@ -665,20 +665,20 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C11" t="n">
-        <v>112.7</v>
+        <v>170.3</v>
       </c>
       <c r="D11" t="n">
-        <v>5.84</v>
+        <v>41.93</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>83.8</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Customer_25 → Customer_23</t>
+          <t>Customer_57 → Customer_60 → Customer_4</t>
         </is>
       </c>
     </row>
@@ -687,20 +687,20 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C12" t="n">
-        <v>170.3</v>
+        <v>224.6</v>
       </c>
       <c r="D12" t="n">
-        <v>41.93</v>
+        <v>46.63</v>
       </c>
       <c r="E12" t="n">
-        <v>83.8</v>
+        <v>52.1</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Customer_57 → Customer_60 → Customer_4</t>
+          <t>Customer_77 → Customer_79 → Customer_37 → Customer_43</t>
         </is>
       </c>
     </row>
@@ -709,20 +709,20 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C13" t="n">
-        <v>270.2</v>
+        <v>246.3</v>
       </c>
       <c r="D13" t="n">
-        <v>74.63</v>
+        <v>83.27</v>
       </c>
       <c r="E13" t="n">
-        <v>57.6</v>
+        <v>51.9</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Customer_77 → Customer_79 → Customer_40 → Customer_44 → Customer_76</t>
+          <t>Customer_21 → Customer_56 → Customer_76 → Customer_44</t>
         </is>
       </c>
     </row>
@@ -734,17 +734,17 @@
         <v>2</v>
       </c>
       <c r="C14" t="n">
-        <v>125.7</v>
+        <v>133.7</v>
       </c>
       <c r="D14" t="n">
-        <v>27.74</v>
+        <v>34.74</v>
       </c>
       <c r="E14" t="n">
-        <v>49.5</v>
+        <v>82.3</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Customer_21 → Customer_56</t>
+          <t>Customer_66 → Customer_13</t>
         </is>
       </c>
     </row>
@@ -753,20 +753,20 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15" t="n">
-        <v>133.7</v>
+        <v>132</v>
       </c>
       <c r="D15" t="n">
-        <v>34.74</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>82.3</v>
+        <v>0</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Customer_66 → Customer_13</t>
+          <t>Customer_20 → Customer_12 → Customer_53</t>
         </is>
       </c>
     </row>
@@ -775,10 +775,10 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>132</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -788,7 +788,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Customer_20 → Customer_12 → Customer_53</t>
+          <t>Customer_5</t>
         </is>
       </c>
     </row>
@@ -800,17 +800,17 @@
         <v>2</v>
       </c>
       <c r="C17" t="n">
-        <v>99</v>
+        <v>124.1</v>
       </c>
       <c r="D17" t="n">
-        <v>7.82</v>
+        <v>24.73</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Customer_43 → Customer_8</t>
+          <t>Customer_40 → Customer_29</t>
         </is>
       </c>
     </row>
@@ -819,20 +819,20 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" t="n">
-        <v>67.09999999999999</v>
+        <v>124.5</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>32.21</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>69.2</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Customer_5</t>
+          <t>Customer_75 → Customer_8</t>
         </is>
       </c>
     </row>
@@ -841,20 +841,20 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>300.6</v>
+        <v>104.5</v>
       </c>
       <c r="D19" t="n">
-        <v>96.76000000000001</v>
+        <v>20.55</v>
       </c>
       <c r="E19" t="n">
-        <v>137.9</v>
+        <v>42.1</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Customer_75 → Customer_63 → Customer_36 → Customer_78</t>
+          <t>Customer_2 → Customer_23</t>
         </is>
       </c>
     </row>
@@ -863,20 +863,20 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>36.2</v>
+        <v>131.3</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>26.61</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>77</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Customer_2</t>
+          <t>Customer_63 → Customer_17</t>
         </is>
       </c>
     </row>
@@ -907,20 +907,20 @@
         <v>20</v>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C22" t="n">
-        <v>50.8</v>
+        <v>135.2</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>36.09</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Customer_28</t>
+          <t>Customer_28 → Customer_78</t>
         </is>
       </c>
     </row>
@@ -929,20 +929,20 @@
         <v>21</v>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C23" t="n">
-        <v>52.7</v>
+        <v>131.1</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>30.69</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Customer_42</t>
+          <t>Customer_42 → Customer_36</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
         <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>34.3</v>
+        <v>49</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
@@ -1007,28 +1007,6 @@
         <v>0</v>
       </c>
       <c r="F26" t="inlineStr">
-        <is>
-          <t>Customer_17</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>25</v>
-      </c>
-      <c r="B27" t="n">
-        <v>1</v>
-      </c>
-      <c r="C27" t="n">
-        <v>49</v>
-      </c>
-      <c r="D27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" t="inlineStr">
         <is>
           <t>Customer_6</t>
         </is>
@@ -1446,16 +1424,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>8117</v>
+        <v>8118</v>
       </c>
       <c r="E8" t="n">
-        <v>314</v>
+        <v>313.8</v>
       </c>
       <c r="F8" t="n">
-        <v>344</v>
+        <v>343.8</v>
       </c>
       <c r="G8" t="n">
-        <v>35.4</v>
+        <v>35.2</v>
       </c>
       <c r="H8" t="n">
         <v>31.6</v>
@@ -1467,20 +1445,24 @@
         <v>11.392</v>
       </c>
       <c r="K8" t="n">
-        <v>254.9</v>
+        <v>282</v>
       </c>
       <c r="L8" t="n">
-        <v>254.9</v>
+        <v>282</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" t="inlineStr"/>
+        <v>27.6</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -2086,13 +2068,13 @@
         <v>15.726</v>
       </c>
       <c r="J20" t="n">
-        <v>49.865</v>
+        <v>49.66</v>
       </c>
       <c r="K20" t="n">
-        <v>268.5</v>
+        <v>268.6</v>
       </c>
       <c r="L20" t="n">
-        <v>268.5</v>
+        <v>268.6</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -2113,45 +2095,49 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Customer_67</t>
+          <t>Customer_31</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2586</v>
+        <v>2596</v>
       </c>
       <c r="E21" t="n">
-        <v>56.6</v>
+        <v>57.9</v>
       </c>
       <c r="F21" t="n">
-        <v>101.6</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="G21" t="n">
-        <v>2.4</v>
+        <v>3.7</v>
       </c>
       <c r="H21" t="n">
-        <v>1.57</v>
+        <v>1.63</v>
       </c>
       <c r="I21" t="n">
-        <v>4.384</v>
+        <v>16.792</v>
       </c>
       <c r="J21" t="n">
-        <v>34.139</v>
+        <v>33.934</v>
       </c>
       <c r="K21" t="n">
-        <v>266</v>
+        <v>282</v>
       </c>
       <c r="L21" t="n">
-        <v>266</v>
+        <v>282</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" t="inlineStr"/>
+        <v>17.4</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2162,45 +2148,49 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Customer_35</t>
+          <t>Customer_67</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>3769</v>
+        <v>1792</v>
       </c>
       <c r="E22" t="n">
-        <v>103.9</v>
+        <v>91.7</v>
       </c>
       <c r="F22" t="n">
-        <v>133.9</v>
+        <v>136.7</v>
       </c>
       <c r="G22" t="n">
-        <v>2.4</v>
+        <v>3.7</v>
       </c>
       <c r="H22" t="n">
-        <v>1.57</v>
+        <v>3.07</v>
       </c>
       <c r="I22" t="n">
-        <v>4.053</v>
+        <v>4.384</v>
       </c>
       <c r="J22" t="n">
-        <v>29.755</v>
+        <v>17.142</v>
       </c>
       <c r="K22" t="n">
-        <v>264</v>
+        <v>282</v>
       </c>
       <c r="L22" t="n">
-        <v>264</v>
+        <v>282</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N22" t="n">
-        <v>0</v>
-      </c>
-      <c r="O22" t="inlineStr"/>
+        <v>4.3</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2215,41 +2205,45 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>2026</v>
+        <v>3803</v>
       </c>
       <c r="E23" t="n">
-        <v>140</v>
+        <v>140.7</v>
       </c>
       <c r="F23" t="n">
-        <v>170</v>
+        <v>170.7</v>
       </c>
       <c r="G23" t="n">
-        <v>6.1</v>
+        <v>4.1</v>
       </c>
       <c r="H23" t="n">
-        <v>5.02</v>
+        <v>3.45</v>
       </c>
       <c r="I23" t="n">
         <v>1.536</v>
       </c>
       <c r="J23" t="n">
-        <v>25.702</v>
+        <v>12.758</v>
       </c>
       <c r="K23" t="n">
-        <v>258</v>
+        <v>282</v>
       </c>
       <c r="L23" t="n">
-        <v>258</v>
+        <v>282</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" t="inlineStr"/>
+        <v>3.4</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2260,84 +2254,90 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Customer_41</t>
+          <t>Customer_18</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>3058</v>
+        <v>8925</v>
       </c>
       <c r="E24" t="n">
-        <v>176.1</v>
+        <v>200.9</v>
       </c>
       <c r="F24" t="n">
-        <v>206.1</v>
+        <v>245.9</v>
       </c>
       <c r="G24" t="n">
-        <v>6.1</v>
+        <v>30.2</v>
       </c>
       <c r="H24" t="n">
-        <v>5.02</v>
+        <v>26.82</v>
       </c>
       <c r="I24" t="n">
-        <v>4.071</v>
+        <v>1.222</v>
       </c>
       <c r="J24" t="n">
-        <v>24.166</v>
+        <v>11.222</v>
       </c>
       <c r="K24" t="n">
-        <v>252.4</v>
+        <v>282</v>
       </c>
       <c r="L24" t="n">
-        <v>252.4</v>
+        <v>282</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" t="inlineStr"/>
+        <v>22.9</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B25" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Customer_16</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>7741</v>
+          <t>Customer_72</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
       </c>
       <c r="E25" t="n">
-        <v>225.3</v>
+        <v>32</v>
       </c>
       <c r="F25" t="n">
-        <v>255.3</v>
+        <v>77</v>
       </c>
       <c r="G25" t="n">
-        <v>19.1</v>
+        <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>15.86</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>4.911</v>
+        <v>9.606</v>
       </c>
       <c r="J25" t="n">
-        <v>20.095</v>
+        <v>49.876</v>
       </c>
       <c r="K25" t="n">
-        <v>235.2</v>
+        <v>235.3</v>
       </c>
       <c r="L25" t="n">
-        <v>235.2</v>
+        <v>235.3</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
@@ -2351,91 +2351,95 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B26" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Customer_9</t>
+          <t>Customer_49</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>5335</v>
+        <v>10890</v>
       </c>
       <c r="E26" t="n">
-        <v>278.3</v>
+        <v>109.8</v>
       </c>
       <c r="F26" t="n">
-        <v>323.3</v>
+        <v>139.8</v>
       </c>
       <c r="G26" t="n">
-        <v>23</v>
+        <v>32.8</v>
       </c>
       <c r="H26" t="n">
-        <v>20.92</v>
+        <v>29.97</v>
       </c>
       <c r="I26" t="n">
-        <v>1.851</v>
+        <v>14.87</v>
       </c>
       <c r="J26" t="n">
-        <v>15.184</v>
+        <v>40.27</v>
       </c>
       <c r="K26" t="n">
-        <v>214.1</v>
+        <v>282</v>
       </c>
       <c r="L26" t="n">
-        <v>214.1</v>
+        <v>282</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" t="inlineStr"/>
+        <v>94.7</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
+        <v>4</v>
+      </c>
+      <c r="B27" t="n">
         <v>3</v>
       </c>
-      <c r="B27" t="n">
-        <v>8</v>
-      </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Customer_59</t>
+          <t>Customer_27</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>11761</v>
+        <v>2754</v>
       </c>
       <c r="E27" t="n">
-        <v>344.3</v>
+        <v>142.1</v>
       </c>
       <c r="F27" t="n">
-        <v>374.3</v>
+        <v>187.1</v>
       </c>
       <c r="G27" t="n">
-        <v>20.9</v>
+        <v>2.3</v>
       </c>
       <c r="H27" t="n">
-        <v>19.15</v>
+        <v>1.52</v>
       </c>
       <c r="I27" t="n">
-        <v>1.454</v>
+        <v>5.276</v>
       </c>
       <c r="J27" t="n">
-        <v>13.333</v>
+        <v>25.4</v>
       </c>
       <c r="K27" t="n">
-        <v>196.7</v>
+        <v>279.9</v>
       </c>
       <c r="L27" t="n">
-        <v>196.7</v>
+        <v>279.9</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -2449,42 +2453,42 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B28" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Customer_62</t>
+          <t>Customer_58</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>3340</v>
+        <v>1543</v>
       </c>
       <c r="E28" t="n">
-        <v>374.3</v>
+        <v>190.6</v>
       </c>
       <c r="F28" t="n">
-        <v>419.3</v>
+        <v>235.6</v>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>3.25</v>
       </c>
       <c r="I28" t="n">
-        <v>1.879</v>
+        <v>1.946</v>
       </c>
       <c r="J28" t="n">
-        <v>11.879</v>
+        <v>20.124</v>
       </c>
       <c r="K28" t="n">
-        <v>196.7</v>
+        <v>276.3</v>
       </c>
       <c r="L28" t="n">
-        <v>196.7</v>
+        <v>276.3</v>
       </c>
       <c r="M28" t="inlineStr">
         <is>
@@ -2501,41 +2505,39 @@
         <v>4</v>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Customer_72</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>VIR</t>
-        </is>
+          <t>Customer_74</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>3291</v>
       </c>
       <c r="E29" t="n">
-        <v>32</v>
+        <v>238.4</v>
       </c>
       <c r="F29" t="n">
-        <v>77</v>
+        <v>268.4</v>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>2.7</v>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>2.51</v>
       </c>
       <c r="I29" t="n">
-        <v>9.606</v>
+        <v>1.146</v>
       </c>
       <c r="J29" t="n">
-        <v>49.149</v>
+        <v>18.178</v>
       </c>
       <c r="K29" t="n">
-        <v>235.7</v>
+        <v>273.8</v>
       </c>
       <c r="L29" t="n">
-        <v>235.7</v>
+        <v>273.8</v>
       </c>
       <c r="M29" t="inlineStr">
         <is>
@@ -2552,33 +2554,33 @@
         <v>4</v>
       </c>
       <c r="B30" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Customer_31</t>
+          <t>Customer_3</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>10863</v>
+        <v>4216</v>
       </c>
       <c r="E30" t="n">
-        <v>100.4</v>
+        <v>280.3</v>
       </c>
       <c r="F30" t="n">
-        <v>130.4</v>
+        <v>325.3</v>
       </c>
       <c r="G30" t="n">
-        <v>23.4</v>
+        <v>12</v>
       </c>
       <c r="H30" t="n">
-        <v>21.08</v>
+        <v>10.24</v>
       </c>
       <c r="I30" t="n">
-        <v>16.792</v>
+        <v>1.503</v>
       </c>
       <c r="J30" t="n">
-        <v>39.543</v>
+        <v>17.032</v>
       </c>
       <c r="K30" t="n">
         <v>282</v>
@@ -2592,11 +2594,11 @@
         </is>
       </c>
       <c r="N30" t="n">
-        <v>80</v>
+        <v>18.8</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -2605,7 +2607,7 @@
         <v>4</v>
       </c>
       <c r="B31" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -2613,188 +2615,184 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1774</v>
+        <v>126</v>
       </c>
       <c r="E31" t="n">
-        <v>134.3</v>
+        <v>331</v>
       </c>
       <c r="F31" t="n">
-        <v>179.3</v>
+        <v>376</v>
       </c>
       <c r="G31" t="n">
-        <v>3.9</v>
+        <v>5.6</v>
       </c>
       <c r="H31" t="n">
-        <v>2.47</v>
+        <v>1.22</v>
       </c>
       <c r="I31" t="n">
         <v>5.529</v>
       </c>
       <c r="J31" t="n">
-        <v>22.751</v>
+        <v>15.529</v>
       </c>
       <c r="K31" t="n">
-        <v>282</v>
+        <v>278.5</v>
       </c>
       <c r="L31" t="n">
-        <v>282</v>
+        <v>278.5</v>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N31" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B32" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Customer_58</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>5188</v>
+          <t>Customer_64</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
       </c>
       <c r="E32" t="n">
-        <v>192.4</v>
+        <v>26.4</v>
       </c>
       <c r="F32" t="n">
-        <v>237.4</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="G32" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>11.08</v>
+        <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>1.946</v>
+        <v>21.424</v>
       </c>
       <c r="J32" t="n">
-        <v>17.222</v>
+        <v>49.308</v>
       </c>
       <c r="K32" t="n">
-        <v>282</v>
+        <v>244.8</v>
       </c>
       <c r="L32" t="n">
-        <v>282</v>
+        <v>244.8</v>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N32" t="n">
-        <v>11.7</v>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B33" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Customer_27</t>
+          <t>Customer_35</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>3297</v>
+        <v>10000</v>
       </c>
       <c r="E33" t="n">
-        <v>240.9</v>
+        <v>90.3</v>
       </c>
       <c r="F33" t="n">
-        <v>285.9</v>
+        <v>120.3</v>
       </c>
       <c r="G33" t="n">
-        <v>3.5</v>
+        <v>18.9</v>
       </c>
       <c r="H33" t="n">
-        <v>3.25</v>
+        <v>15.86</v>
       </c>
       <c r="I33" t="n">
-        <v>5.276</v>
+        <v>4.053</v>
       </c>
       <c r="J33" t="n">
-        <v>15.276</v>
+        <v>27.884</v>
       </c>
       <c r="K33" t="n">
-        <v>278.9</v>
+        <v>282</v>
       </c>
       <c r="L33" t="n">
-        <v>278.9</v>
+        <v>282</v>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N33" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" t="inlineStr"/>
+        <v>63.4</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
         <v>5</v>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Customer_64</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>VIR</t>
-        </is>
+          <t>Customer_16</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>7182</v>
       </c>
       <c r="E34" t="n">
-        <v>26.4</v>
+        <v>139.5</v>
       </c>
       <c r="F34" t="n">
-        <v>71.40000000000001</v>
+        <v>169.5</v>
       </c>
       <c r="G34" t="n">
-        <v>0</v>
+        <v>19.1</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>15.86</v>
       </c>
       <c r="I34" t="n">
-        <v>21.424</v>
+        <v>4.911</v>
       </c>
       <c r="J34" t="n">
-        <v>49.689</v>
+        <v>23.831</v>
       </c>
       <c r="K34" t="n">
-        <v>244.6</v>
+        <v>263.6</v>
       </c>
       <c r="L34" t="n">
-        <v>244.6</v>
+        <v>263.6</v>
       </c>
       <c r="M34" t="inlineStr">
         <is>
@@ -2811,33 +2809,33 @@
         <v>5</v>
       </c>
       <c r="B35" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Customer_48</t>
+          <t>Customer_41</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>10022</v>
+        <v>5275</v>
       </c>
       <c r="E35" t="n">
-        <v>97.59999999999999</v>
+        <v>188.4</v>
       </c>
       <c r="F35" t="n">
-        <v>127.6</v>
+        <v>218.4</v>
       </c>
       <c r="G35" t="n">
-        <v>26.2</v>
+        <v>18.9</v>
       </c>
       <c r="H35" t="n">
-        <v>23.1</v>
+        <v>15.86</v>
       </c>
       <c r="I35" t="n">
-        <v>3.395</v>
+        <v>4.071</v>
       </c>
       <c r="J35" t="n">
-        <v>28.265</v>
+        <v>18.92</v>
       </c>
       <c r="K35" t="n">
         <v>282</v>
@@ -2851,11 +2849,11 @@
         </is>
       </c>
       <c r="N35" t="n">
-        <v>74.2</v>
+        <v>36.1</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -2864,143 +2862,143 @@
         <v>5</v>
       </c>
       <c r="B36" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Customer_49</t>
+          <t>Customer_48</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>8329</v>
+        <v>7771</v>
       </c>
       <c r="E36" t="n">
-        <v>142.9</v>
+        <v>227.1</v>
       </c>
       <c r="F36" t="n">
-        <v>172.9</v>
+        <v>257.1</v>
       </c>
       <c r="G36" t="n">
-        <v>15.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H36" t="n">
-        <v>14.08</v>
+        <v>8.01</v>
       </c>
       <c r="I36" t="n">
-        <v>14.87</v>
+        <v>3.395</v>
       </c>
       <c r="J36" t="n">
-        <v>24.87</v>
+        <v>14.849</v>
       </c>
       <c r="K36" t="n">
-        <v>282</v>
+        <v>274.2</v>
       </c>
       <c r="L36" t="n">
-        <v>282</v>
+        <v>274.2</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N36" t="n">
-        <v>16.4</v>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
+        <v>5</v>
+      </c>
+      <c r="B37" t="n">
         <v>6</v>
       </c>
-      <c r="B37" t="n">
-        <v>1</v>
-      </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Customer_30</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>VIR</t>
-        </is>
+          <t>Customer_59</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>8340</v>
       </c>
       <c r="E37" t="n">
-        <v>10.3</v>
+        <v>297.5</v>
       </c>
       <c r="F37" t="n">
-        <v>55.3</v>
+        <v>327.5</v>
       </c>
       <c r="G37" t="n">
-        <v>0</v>
+        <v>40.4</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>37.02</v>
       </c>
       <c r="I37" t="n">
-        <v>34.69</v>
+        <v>1.454</v>
       </c>
       <c r="J37" t="n">
-        <v>49.298</v>
+        <v>11.454</v>
       </c>
       <c r="K37" t="n">
-        <v>268.4</v>
+        <v>282</v>
       </c>
       <c r="L37" t="n">
-        <v>268.4</v>
+        <v>282</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N37" t="n">
-        <v>0</v>
-      </c>
-      <c r="O37" t="inlineStr"/>
+        <v>41</v>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
         <v>6</v>
       </c>
       <c r="B38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Customer_73</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>1749</v>
+          <t>Customer_30</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
       </c>
       <c r="E38" t="n">
-        <v>65.59999999999999</v>
+        <v>10.3</v>
       </c>
       <c r="F38" t="n">
-        <v>95.59999999999999</v>
+        <v>55.3</v>
       </c>
       <c r="G38" t="n">
-        <v>10.4</v>
+        <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>9.51</v>
+        <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>4.608</v>
+        <v>34.69</v>
       </c>
       <c r="J38" t="n">
-        <v>14.608</v>
+        <v>49.298</v>
       </c>
       <c r="K38" t="n">
-        <v>253.3</v>
+        <v>268.4</v>
       </c>
       <c r="L38" t="n">
-        <v>253.3</v>
+        <v>268.4</v>
       </c>
       <c r="M38" t="inlineStr">
         <is>
@@ -3014,44 +3012,42 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Customer_18</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>VIR</t>
-        </is>
+          <t>Customer_73</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1749</v>
       </c>
       <c r="E39" t="n">
-        <v>20.8</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="F39" t="n">
-        <v>65.8</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="G39" t="n">
-        <v>0</v>
+        <v>10.4</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>9.51</v>
       </c>
       <c r="I39" t="n">
-        <v>1.222</v>
+        <v>4.608</v>
       </c>
       <c r="J39" t="n">
-        <v>49.431</v>
+        <v>14.608</v>
       </c>
       <c r="K39" t="n">
-        <v>252</v>
+        <v>253.3</v>
       </c>
       <c r="L39" t="n">
-        <v>252</v>
+        <v>253.3</v>
       </c>
       <c r="M39" t="inlineStr">
         <is>
@@ -3068,86 +3064,84 @@
         <v>7</v>
       </c>
       <c r="B40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Customer_29</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>5453</v>
+          <t>Customer_22</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
       </c>
       <c r="E40" t="n">
-        <v>92.40000000000001</v>
+        <v>4.6</v>
       </c>
       <c r="F40" t="n">
-        <v>137.4</v>
+        <v>49.6</v>
       </c>
       <c r="G40" t="n">
-        <v>26.7</v>
+        <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>23.42</v>
+        <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>32.083</v>
+        <v>22.317</v>
       </c>
       <c r="J40" t="n">
-        <v>48.209</v>
+        <v>49.807</v>
       </c>
       <c r="K40" t="n">
-        <v>282</v>
+        <v>275.2</v>
       </c>
       <c r="L40" t="n">
-        <v>282</v>
+        <v>275.2</v>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N40" t="n">
-        <v>68.59999999999999</v>
-      </c>
-      <c r="O40" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
         <v>7</v>
       </c>
       <c r="B41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Customer_3</t>
+          <t>Customer_7</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1668</v>
+        <v>5960</v>
       </c>
       <c r="E41" t="n">
-        <v>143.2</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="F41" t="n">
-        <v>188.2</v>
+        <v>118.6</v>
       </c>
       <c r="G41" t="n">
-        <v>5.7</v>
+        <v>24</v>
       </c>
       <c r="H41" t="n">
-        <v>2.88</v>
+        <v>21.97</v>
       </c>
       <c r="I41" t="n">
-        <v>1.503</v>
+        <v>14.668</v>
       </c>
       <c r="J41" t="n">
-        <v>16.126</v>
+        <v>27.49</v>
       </c>
       <c r="K41" t="n">
         <v>282</v>
@@ -3161,11 +3155,11 @@
         </is>
       </c>
       <c r="N41" t="n">
-        <v>7.2</v>
+        <v>41.9</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -3174,145 +3168,139 @@
         <v>7</v>
       </c>
       <c r="B42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Customer_11</t>
+          <t>Customer_39</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>6692</v>
+        <v>10603</v>
       </c>
       <c r="E42" t="n">
-        <v>209.8</v>
+        <v>146.7</v>
       </c>
       <c r="F42" t="n">
-        <v>239.8</v>
+        <v>176.7</v>
       </c>
       <c r="G42" t="n">
-        <v>21.6</v>
+        <v>28.1</v>
       </c>
       <c r="H42" t="n">
-        <v>19.32</v>
+        <v>25.78</v>
       </c>
       <c r="I42" t="n">
-        <v>1.696</v>
+        <v>1.781</v>
       </c>
       <c r="J42" t="n">
-        <v>14.623</v>
+        <v>12.822</v>
       </c>
       <c r="K42" t="n">
-        <v>282</v>
+        <v>252.4</v>
       </c>
       <c r="L42" t="n">
-        <v>282</v>
+        <v>252.4</v>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N42" t="n">
-        <v>18.1</v>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
         <v>7</v>
       </c>
       <c r="B43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Customer_74</t>
+          <t>Customer_61</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>4852</v>
+        <v>7546</v>
       </c>
       <c r="E43" t="n">
-        <v>270.2</v>
+        <v>223.4</v>
       </c>
       <c r="F43" t="n">
-        <v>300.2</v>
+        <v>268.4</v>
       </c>
       <c r="G43" t="n">
-        <v>30.5</v>
+        <v>46.6</v>
       </c>
       <c r="H43" t="n">
-        <v>27.83</v>
+        <v>42.75</v>
       </c>
       <c r="I43" t="n">
-        <v>1.146</v>
+        <v>1.041</v>
       </c>
       <c r="J43" t="n">
-        <v>12.927</v>
+        <v>11.041</v>
       </c>
       <c r="K43" t="n">
-        <v>282</v>
+        <v>215.8</v>
       </c>
       <c r="L43" t="n">
-        <v>282</v>
+        <v>215.8</v>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N43" t="n">
-        <v>24.9</v>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B44" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Customer_39</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
-        <v>4200</v>
+          <t>Customer_25</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
       </c>
       <c r="E44" t="n">
-        <v>310.1</v>
+        <v>30.6</v>
       </c>
       <c r="F44" t="n">
-        <v>340.1</v>
+        <v>60.6</v>
       </c>
       <c r="G44" t="n">
-        <v>9.9</v>
+        <v>0</v>
       </c>
       <c r="H44" t="n">
-        <v>9.07</v>
+        <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>1.781</v>
+        <v>33.124</v>
       </c>
       <c r="J44" t="n">
-        <v>11.781</v>
+        <v>48.55</v>
       </c>
       <c r="K44" t="n">
-        <v>274.2</v>
+        <v>239.2</v>
       </c>
       <c r="L44" t="n">
-        <v>274.2</v>
+        <v>239.2</v>
       </c>
       <c r="M44" t="inlineStr">
         <is>
@@ -3329,41 +3317,39 @@
         <v>8</v>
       </c>
       <c r="B45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Customer_22</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>VIR</t>
-        </is>
+          <t>Customer_9</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>6303</v>
       </c>
       <c r="E45" t="n">
-        <v>4.6</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="F45" t="n">
-        <v>49.6</v>
+        <v>128.9</v>
       </c>
       <c r="G45" t="n">
-        <v>0</v>
+        <v>23.4</v>
       </c>
       <c r="H45" t="n">
-        <v>0</v>
+        <v>21.23</v>
       </c>
       <c r="I45" t="n">
-        <v>22.317</v>
+        <v>1.851</v>
       </c>
       <c r="J45" t="n">
-        <v>49.802</v>
+        <v>15.426</v>
       </c>
       <c r="K45" t="n">
-        <v>275.2</v>
+        <v>205.5</v>
       </c>
       <c r="L45" t="n">
-        <v>275.2</v>
+        <v>205.5</v>
       </c>
       <c r="M45" t="inlineStr">
         <is>
@@ -3380,92 +3366,88 @@
         <v>8</v>
       </c>
       <c r="B46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Customer_7</t>
+          <t>Customer_62</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>5960</v>
+        <v>11767</v>
       </c>
       <c r="E46" t="n">
-        <v>73.59999999999999</v>
+        <v>149.9</v>
       </c>
       <c r="F46" t="n">
-        <v>118.6</v>
+        <v>194.9</v>
       </c>
       <c r="G46" t="n">
-        <v>24</v>
+        <v>20.9</v>
       </c>
       <c r="H46" t="n">
-        <v>21.97</v>
+        <v>19.15</v>
       </c>
       <c r="I46" t="n">
-        <v>14.668</v>
+        <v>1.879</v>
       </c>
       <c r="J46" t="n">
-        <v>27.485</v>
+        <v>13.575</v>
       </c>
       <c r="K46" t="n">
-        <v>282</v>
+        <v>188</v>
       </c>
       <c r="L46" t="n">
-        <v>282</v>
+        <v>188</v>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N46" t="n">
-        <v>41.9</v>
-      </c>
-      <c r="O46" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
         <v>8</v>
       </c>
       <c r="B47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Customer_37</t>
+          <t>Customer_11</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>360</v>
+        <v>9774</v>
       </c>
       <c r="E47" t="n">
-        <v>121.7</v>
+        <v>227.9</v>
       </c>
       <c r="F47" t="n">
-        <v>166.7</v>
+        <v>257.9</v>
       </c>
       <c r="G47" t="n">
-        <v>3.1</v>
+        <v>33</v>
       </c>
       <c r="H47" t="n">
-        <v>2.83</v>
+        <v>30.11</v>
       </c>
       <c r="I47" t="n">
-        <v>1.776</v>
+        <v>1.696</v>
       </c>
       <c r="J47" t="n">
-        <v>12.817</v>
+        <v>11.696</v>
       </c>
       <c r="K47" t="n">
-        <v>278.7</v>
+        <v>161.7</v>
       </c>
       <c r="L47" t="n">
-        <v>278.7</v>
+        <v>161.7</v>
       </c>
       <c r="M47" t="inlineStr">
         <is>
@@ -3479,42 +3461,44 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B48" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Customer_61</t>
-        </is>
-      </c>
-      <c r="D48" t="n">
-        <v>7377</v>
+          <t>Customer_57</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
       </c>
       <c r="E48" t="n">
-        <v>188.4</v>
+        <v>18.6</v>
       </c>
       <c r="F48" t="n">
-        <v>233.4</v>
+        <v>48.6</v>
       </c>
       <c r="G48" t="n">
-        <v>21.7</v>
+        <v>0</v>
       </c>
       <c r="H48" t="n">
-        <v>19.91</v>
+        <v>0</v>
       </c>
       <c r="I48" t="n">
-        <v>1.041</v>
+        <v>29.692</v>
       </c>
       <c r="J48" t="n">
-        <v>11.041</v>
+        <v>49.218</v>
       </c>
       <c r="K48" t="n">
-        <v>261.7</v>
+        <v>255</v>
       </c>
       <c r="L48" t="n">
-        <v>261.7</v>
+        <v>255</v>
       </c>
       <c r="M48" t="inlineStr">
         <is>
@@ -3531,100 +3515,106 @@
         <v>9</v>
       </c>
       <c r="B49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Customer_25</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>VIR</t>
-        </is>
+          <t>Customer_60</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>9280</v>
       </c>
       <c r="E49" t="n">
-        <v>30.6</v>
+        <v>77.5</v>
       </c>
       <c r="F49" t="n">
-        <v>60.6</v>
+        <v>122.5</v>
       </c>
       <c r="G49" t="n">
-        <v>0</v>
+        <v>28.9</v>
       </c>
       <c r="H49" t="n">
-        <v>0</v>
+        <v>25.62</v>
       </c>
       <c r="I49" t="n">
-        <v>33.124</v>
+        <v>4.369</v>
       </c>
       <c r="J49" t="n">
-        <v>48.791</v>
+        <v>19.526</v>
       </c>
       <c r="K49" t="n">
-        <v>239</v>
+        <v>282</v>
       </c>
       <c r="L49" t="n">
-        <v>239</v>
+        <v>282</v>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N49" t="n">
-        <v>0</v>
-      </c>
-      <c r="O49" t="inlineStr"/>
+        <v>67.59999999999999</v>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
         <v>9</v>
       </c>
       <c r="B50" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Customer_23</t>
+          <t>Customer_4</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1423</v>
+        <v>9606</v>
       </c>
       <c r="E50" t="n">
-        <v>67.7</v>
+        <v>140.3</v>
       </c>
       <c r="F50" t="n">
-        <v>112.7</v>
+        <v>170.3</v>
       </c>
       <c r="G50" t="n">
-        <v>7.1</v>
+        <v>17.8</v>
       </c>
       <c r="H50" t="n">
-        <v>5.84</v>
+        <v>16.32</v>
       </c>
       <c r="I50" t="n">
-        <v>5.667</v>
+        <v>5.157</v>
       </c>
       <c r="J50" t="n">
-        <v>15.667</v>
+        <v>15.157</v>
       </c>
       <c r="K50" t="n">
-        <v>228.7</v>
+        <v>282</v>
       </c>
       <c r="L50" t="n">
-        <v>228.7</v>
+        <v>282</v>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N50" t="n">
-        <v>0</v>
-      </c>
-      <c r="O50" t="inlineStr"/>
+        <v>16.2</v>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -3635,7 +3625,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Customer_57</t>
+          <t>Customer_77</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3644,10 +3634,10 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>18.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F51" t="n">
-        <v>48.6</v>
+        <v>53.8</v>
       </c>
       <c r="G51" t="n">
         <v>0</v>
@@ -3656,16 +3646,16 @@
         <v>0</v>
       </c>
       <c r="I51" t="n">
-        <v>29.692</v>
+        <v>20.562</v>
       </c>
       <c r="J51" t="n">
-        <v>49.218</v>
+        <v>48.775</v>
       </c>
       <c r="K51" t="n">
-        <v>255</v>
+        <v>269.3</v>
       </c>
       <c r="L51" t="n">
-        <v>255</v>
+        <v>269.3</v>
       </c>
       <c r="M51" t="inlineStr">
         <is>
@@ -3686,29 +3676,29 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Customer_60</t>
+          <t>Customer_79</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>9280</v>
+        <v>11331</v>
       </c>
       <c r="E52" t="n">
-        <v>77.5</v>
+        <v>65.8</v>
       </c>
       <c r="F52" t="n">
-        <v>122.5</v>
+        <v>110.8</v>
       </c>
       <c r="G52" t="n">
-        <v>28.9</v>
+        <v>12.1</v>
       </c>
       <c r="H52" t="n">
-        <v>25.62</v>
+        <v>11.06</v>
       </c>
       <c r="I52" t="n">
-        <v>4.369</v>
+        <v>10.495</v>
       </c>
       <c r="J52" t="n">
-        <v>19.526</v>
+        <v>28.213</v>
       </c>
       <c r="K52" t="n">
         <v>282</v>
@@ -3722,7 +3712,7 @@
         </is>
       </c>
       <c r="N52" t="n">
-        <v>67.59999999999999</v>
+        <v>30.1</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
@@ -3739,29 +3729,29 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Customer_4</t>
+          <t>Customer_37</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>9606</v>
+        <v>11447</v>
       </c>
       <c r="E53" t="n">
-        <v>140.3</v>
+        <v>131.5</v>
       </c>
       <c r="F53" t="n">
-        <v>170.3</v>
+        <v>176.5</v>
       </c>
       <c r="G53" t="n">
-        <v>17.8</v>
+        <v>20.7</v>
       </c>
       <c r="H53" t="n">
-        <v>16.32</v>
+        <v>18.96</v>
       </c>
       <c r="I53" t="n">
-        <v>5.157</v>
+        <v>1.776</v>
       </c>
       <c r="J53" t="n">
-        <v>15.157</v>
+        <v>17.718</v>
       </c>
       <c r="K53" t="n">
         <v>282</v>
@@ -3775,54 +3765,52 @@
         </is>
       </c>
       <c r="N53" t="n">
-        <v>16.2</v>
+        <v>22.1</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B54" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Customer_77</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>VIR</t>
-        </is>
+          <t>Customer_43</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>7361</v>
       </c>
       <c r="E54" t="n">
-        <v>8.800000000000001</v>
+        <v>194.6</v>
       </c>
       <c r="F54" t="n">
-        <v>53.8</v>
+        <v>224.6</v>
       </c>
       <c r="G54" t="n">
-        <v>0</v>
+        <v>18.1</v>
       </c>
       <c r="H54" t="n">
-        <v>0</v>
+        <v>16.61</v>
       </c>
       <c r="I54" t="n">
-        <v>20.562</v>
+        <v>5.942</v>
       </c>
       <c r="J54" t="n">
-        <v>49.253</v>
+        <v>15.942</v>
       </c>
       <c r="K54" t="n">
-        <v>269.3</v>
+        <v>266.2</v>
       </c>
       <c r="L54" t="n">
-        <v>269.3</v>
+        <v>266.2</v>
       </c>
       <c r="M54" t="inlineStr">
         <is>
@@ -3839,86 +3827,84 @@
         <v>11</v>
       </c>
       <c r="B55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Customer_79</t>
-        </is>
-      </c>
-      <c r="D55" t="n">
-        <v>11331</v>
+          <t>Customer_21</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
       </c>
       <c r="E55" t="n">
-        <v>65.8</v>
+        <v>4.6</v>
       </c>
       <c r="F55" t="n">
-        <v>110.8</v>
+        <v>49.6</v>
       </c>
       <c r="G55" t="n">
-        <v>12.1</v>
+        <v>0</v>
       </c>
       <c r="H55" t="n">
-        <v>11.06</v>
+        <v>0</v>
       </c>
       <c r="I55" t="n">
-        <v>10.495</v>
+        <v>26.403</v>
       </c>
       <c r="J55" t="n">
-        <v>28.691</v>
+        <v>49.329</v>
       </c>
       <c r="K55" t="n">
-        <v>282</v>
+        <v>275.2</v>
       </c>
       <c r="L55" t="n">
-        <v>282</v>
+        <v>275.2</v>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N55" t="n">
-        <v>30.3</v>
-      </c>
-      <c r="O55" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
         <v>11</v>
       </c>
       <c r="B56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Customer_40</t>
+          <t>Customer_56</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>11450</v>
+        <v>5851</v>
       </c>
       <c r="E56" t="n">
-        <v>136.3</v>
+        <v>80.7</v>
       </c>
       <c r="F56" t="n">
-        <v>166.3</v>
+        <v>125.7</v>
       </c>
       <c r="G56" t="n">
-        <v>25.4</v>
+        <v>31.1</v>
       </c>
       <c r="H56" t="n">
-        <v>23.31</v>
+        <v>27.74</v>
       </c>
       <c r="I56" t="n">
-        <v>4.524</v>
+        <v>9.254</v>
       </c>
       <c r="J56" t="n">
-        <v>18.196</v>
+        <v>22.926</v>
       </c>
       <c r="K56" t="n">
         <v>282</v>
@@ -3932,7 +3918,7 @@
         </is>
       </c>
       <c r="N56" t="n">
-        <v>27.4</v>
+        <v>51.9</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
@@ -3945,39 +3931,39 @@
         <v>11</v>
       </c>
       <c r="B57" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Customer_44</t>
+          <t>Customer_76</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>2282</v>
+        <v>9219</v>
       </c>
       <c r="E57" t="n">
-        <v>166.3</v>
+        <v>142.4</v>
       </c>
       <c r="F57" t="n">
-        <v>196.3</v>
+        <v>172.4</v>
       </c>
       <c r="G57" t="n">
-        <v>0</v>
+        <v>16.7</v>
       </c>
       <c r="H57" t="n">
-        <v>0</v>
+        <v>15.27</v>
       </c>
       <c r="I57" t="n">
-        <v>1.975</v>
+        <v>1.697</v>
       </c>
       <c r="J57" t="n">
         <v>13.672</v>
       </c>
       <c r="K57" t="n">
-        <v>282</v>
+        <v>265.8</v>
       </c>
       <c r="L57" t="n">
-        <v>282</v>
+        <v>265.8</v>
       </c>
       <c r="M57" t="inlineStr">
         <is>
@@ -3994,21 +3980,21 @@
         <v>11</v>
       </c>
       <c r="B58" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Customer_76</t>
+          <t>Customer_44</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>8061</v>
+        <v>11218</v>
       </c>
       <c r="E58" t="n">
-        <v>240.2</v>
+        <v>216.3</v>
       </c>
       <c r="F58" t="n">
-        <v>270.2</v>
+        <v>246.3</v>
       </c>
       <c r="G58" t="n">
         <v>43.9</v>
@@ -4017,16 +4003,16 @@
         <v>40.26</v>
       </c>
       <c r="I58" t="n">
-        <v>1.697</v>
+        <v>1.975</v>
       </c>
       <c r="J58" t="n">
-        <v>11.697</v>
+        <v>11.975</v>
       </c>
       <c r="K58" t="n">
-        <v>246.8</v>
+        <v>230.7</v>
       </c>
       <c r="L58" t="n">
-        <v>246.8</v>
+        <v>230.7</v>
       </c>
       <c r="M58" t="inlineStr">
         <is>
@@ -4047,7 +4033,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Customer_21</t>
+          <t>Customer_66</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -4056,10 +4042,10 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>4.6</v>
+        <v>20.8</v>
       </c>
       <c r="F59" t="n">
-        <v>49.6</v>
+        <v>50.8</v>
       </c>
       <c r="G59" t="n">
         <v>0</v>
@@ -4068,16 +4054,16 @@
         <v>0</v>
       </c>
       <c r="I59" t="n">
-        <v>26.403</v>
+        <v>30.607</v>
       </c>
       <c r="J59" t="n">
-        <v>45.657</v>
+        <v>46.485</v>
       </c>
       <c r="K59" t="n">
-        <v>275.6</v>
+        <v>252.9</v>
       </c>
       <c r="L59" t="n">
-        <v>275.6</v>
+        <v>252.9</v>
       </c>
       <c r="M59" t="inlineStr">
         <is>
@@ -4098,29 +4084,29 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Customer_56</t>
+          <t>Customer_13</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>5851</v>
+        <v>10170</v>
       </c>
       <c r="E60" t="n">
-        <v>80.7</v>
+        <v>88.7</v>
       </c>
       <c r="F60" t="n">
-        <v>125.7</v>
+        <v>133.7</v>
       </c>
       <c r="G60" t="n">
-        <v>31.1</v>
+        <v>37.9</v>
       </c>
       <c r="H60" t="n">
-        <v>27.74</v>
+        <v>34.74</v>
       </c>
       <c r="I60" t="n">
-        <v>9.254</v>
+        <v>5.878</v>
       </c>
       <c r="J60" t="n">
-        <v>19.254</v>
+        <v>15.878</v>
       </c>
       <c r="K60" t="n">
         <v>282</v>
@@ -4134,7 +4120,7 @@
         </is>
       </c>
       <c r="N60" t="n">
-        <v>49.5</v>
+        <v>82.3</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
@@ -4151,7 +4137,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Customer_66</t>
+          <t>Customer_20</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -4160,10 +4146,10 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>20.8</v>
+        <v>27</v>
       </c>
       <c r="F61" t="n">
-        <v>50.8</v>
+        <v>72</v>
       </c>
       <c r="G61" t="n">
         <v>0</v>
@@ -4172,16 +4158,16 @@
         <v>0</v>
       </c>
       <c r="I61" t="n">
-        <v>30.607</v>
+        <v>23.057</v>
       </c>
       <c r="J61" t="n">
-        <v>46.485</v>
+        <v>49.191</v>
       </c>
       <c r="K61" t="n">
-        <v>252.9</v>
+        <v>242.9</v>
       </c>
       <c r="L61" t="n">
-        <v>252.9</v>
+        <v>242.9</v>
       </c>
       <c r="M61" t="inlineStr">
         <is>
@@ -4202,72 +4188,66 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Customer_13</t>
+          <t>Customer_12</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>10170</v>
+        <v>1118</v>
       </c>
       <c r="E62" t="n">
-        <v>88.7</v>
+        <v>72</v>
       </c>
       <c r="F62" t="n">
-        <v>133.7</v>
+        <v>102</v>
       </c>
       <c r="G62" t="n">
-        <v>37.9</v>
+        <v>0</v>
       </c>
       <c r="H62" t="n">
-        <v>34.74</v>
+        <v>0</v>
       </c>
       <c r="I62" t="n">
-        <v>5.878</v>
+        <v>4.396</v>
       </c>
       <c r="J62" t="n">
-        <v>15.878</v>
+        <v>26.134</v>
       </c>
       <c r="K62" t="n">
-        <v>282</v>
+        <v>242.9</v>
       </c>
       <c r="L62" t="n">
-        <v>282</v>
+        <v>242.9</v>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N62" t="n">
-        <v>82.3</v>
-      </c>
-      <c r="O62" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B63" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Customer_20</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>VIR</t>
-        </is>
+          <t>Customer_53</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>656</v>
       </c>
       <c r="E63" t="n">
-        <v>27</v>
+        <v>102</v>
       </c>
       <c r="F63" t="n">
-        <v>72</v>
+        <v>132</v>
       </c>
       <c r="G63" t="n">
         <v>0</v>
@@ -4276,10 +4256,10 @@
         <v>0</v>
       </c>
       <c r="I63" t="n">
-        <v>23.057</v>
+        <v>11.738</v>
       </c>
       <c r="J63" t="n">
-        <v>49.191</v>
+        <v>21.738</v>
       </c>
       <c r="K63" t="n">
         <v>242.9</v>
@@ -4302,21 +4282,23 @@
         <v>14</v>
       </c>
       <c r="B64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Customer_12</t>
-        </is>
-      </c>
-      <c r="D64" t="n">
-        <v>1118</v>
+          <t>Customer_5</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
       </c>
       <c r="E64" t="n">
-        <v>72</v>
+        <v>22.1</v>
       </c>
       <c r="F64" t="n">
-        <v>102</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="G64" t="n">
         <v>0</v>
@@ -4325,16 +4307,16 @@
         <v>0</v>
       </c>
       <c r="I64" t="n">
-        <v>4.396</v>
+        <v>35.722</v>
       </c>
       <c r="J64" t="n">
-        <v>26.134</v>
+        <v>45.722</v>
       </c>
       <c r="K64" t="n">
-        <v>242.9</v>
+        <v>252</v>
       </c>
       <c r="L64" t="n">
-        <v>242.9</v>
+        <v>252</v>
       </c>
       <c r="M64" t="inlineStr">
         <is>
@@ -4348,24 +4330,26 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B65" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Customer_53</t>
-        </is>
-      </c>
-      <c r="D65" t="n">
-        <v>656</v>
+          <t>Customer_40</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
       </c>
       <c r="E65" t="n">
-        <v>102</v>
+        <v>22.1</v>
       </c>
       <c r="F65" t="n">
-        <v>132</v>
+        <v>52.1</v>
       </c>
       <c r="G65" t="n">
         <v>0</v>
@@ -4374,16 +4358,16 @@
         <v>0</v>
       </c>
       <c r="I65" t="n">
-        <v>11.738</v>
+        <v>4.524</v>
       </c>
       <c r="J65" t="n">
-        <v>21.738</v>
+        <v>46.607</v>
       </c>
       <c r="K65" t="n">
-        <v>242.9</v>
+        <v>250.9</v>
       </c>
       <c r="L65" t="n">
-        <v>242.9</v>
+        <v>250.9</v>
       </c>
       <c r="M65" t="inlineStr">
         <is>
@@ -4400,41 +4384,39 @@
         <v>15</v>
       </c>
       <c r="B66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Customer_43</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>VIR</t>
-        </is>
+          <t>Customer_29</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>7674</v>
       </c>
       <c r="E66" t="n">
-        <v>30.5</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="F66" t="n">
-        <v>60.5</v>
+        <v>124.1</v>
       </c>
       <c r="G66" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="H66" t="n">
-        <v>0</v>
+        <v>24.73</v>
       </c>
       <c r="I66" t="n">
-        <v>5.942</v>
+        <v>32.083</v>
       </c>
       <c r="J66" t="n">
-        <v>47.492</v>
+        <v>42.083</v>
       </c>
       <c r="K66" t="n">
-        <v>238.9</v>
+        <v>213</v>
       </c>
       <c r="L66" t="n">
-        <v>238.9</v>
+        <v>213</v>
       </c>
       <c r="M66" t="inlineStr">
         <is>
@@ -4448,42 +4430,44 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Customer_8</t>
-        </is>
-      </c>
-      <c r="D67" t="n">
-        <v>2447</v>
+          <t>Customer_75</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
       </c>
       <c r="E67" t="n">
-        <v>69</v>
+        <v>14.2</v>
       </c>
       <c r="F67" t="n">
-        <v>99</v>
+        <v>59.2</v>
       </c>
       <c r="G67" t="n">
-        <v>8.5</v>
+        <v>0</v>
       </c>
       <c r="H67" t="n">
-        <v>7.82</v>
+        <v>0</v>
       </c>
       <c r="I67" t="n">
-        <v>31.55</v>
+        <v>4.741</v>
       </c>
       <c r="J67" t="n">
-        <v>41.55</v>
+        <v>46.291</v>
       </c>
       <c r="K67" t="n">
-        <v>226.8</v>
+        <v>262.1</v>
       </c>
       <c r="L67" t="n">
-        <v>226.8</v>
+        <v>262.1</v>
       </c>
       <c r="M67" t="inlineStr">
         <is>
@@ -4500,51 +4484,53 @@
         <v>16</v>
       </c>
       <c r="B68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Customer_5</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>VIR</t>
-        </is>
+          <t>Customer_8</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>11164</v>
       </c>
       <c r="E68" t="n">
-        <v>22.1</v>
+        <v>94.5</v>
       </c>
       <c r="F68" t="n">
-        <v>67.09999999999999</v>
+        <v>124.5</v>
       </c>
       <c r="G68" t="n">
-        <v>0</v>
+        <v>35.2</v>
       </c>
       <c r="H68" t="n">
-        <v>0</v>
+        <v>32.21</v>
       </c>
       <c r="I68" t="n">
-        <v>35.722</v>
+        <v>31.55</v>
       </c>
       <c r="J68" t="n">
-        <v>45.722</v>
+        <v>41.55</v>
       </c>
       <c r="K68" t="n">
-        <v>252</v>
+        <v>282</v>
       </c>
       <c r="L68" t="n">
-        <v>252</v>
+        <v>282</v>
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N68" t="n">
-        <v>0</v>
-      </c>
-      <c r="O68" t="inlineStr"/>
+        <v>69.2</v>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -4555,7 +4541,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Customer_75</t>
+          <t>Customer_2</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -4564,10 +4550,10 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>14.2</v>
+        <v>6.2</v>
       </c>
       <c r="F69" t="n">
-        <v>59.2</v>
+        <v>36.2</v>
       </c>
       <c r="G69" t="n">
         <v>0</v>
@@ -4576,16 +4562,16 @@
         <v>0</v>
       </c>
       <c r="I69" t="n">
-        <v>4.741</v>
+        <v>32.335</v>
       </c>
       <c r="J69" t="n">
-        <v>38.289</v>
+        <v>48.002</v>
       </c>
       <c r="K69" t="n">
-        <v>264.2</v>
+        <v>273.2</v>
       </c>
       <c r="L69" t="n">
-        <v>264.2</v>
+        <v>273.2</v>
       </c>
       <c r="M69" t="inlineStr">
         <is>
@@ -4606,29 +4592,29 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Customer_63</t>
+          <t>Customer_23</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>11147</v>
+        <v>5626</v>
       </c>
       <c r="E70" t="n">
-        <v>99</v>
+        <v>59.5</v>
       </c>
       <c r="F70" t="n">
-        <v>144</v>
+        <v>104.5</v>
       </c>
       <c r="G70" t="n">
-        <v>39.7</v>
+        <v>23.3</v>
       </c>
       <c r="H70" t="n">
-        <v>35.68</v>
+        <v>20.55</v>
       </c>
       <c r="I70" t="n">
-        <v>8.436999999999999</v>
+        <v>5.667</v>
       </c>
       <c r="J70" t="n">
-        <v>33.548</v>
+        <v>15.667</v>
       </c>
       <c r="K70" t="n">
         <v>282</v>
@@ -4642,7 +4628,7 @@
         </is>
       </c>
       <c r="N70" t="n">
-        <v>67.5</v>
+        <v>42.1</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
@@ -4652,42 +4638,44 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B71" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Customer_36</t>
-        </is>
-      </c>
-      <c r="D71" t="n">
-        <v>9890</v>
+          <t>Customer_63</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
       </c>
       <c r="E71" t="n">
-        <v>163.7</v>
+        <v>26.4</v>
       </c>
       <c r="F71" t="n">
-        <v>208.7</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="G71" t="n">
-        <v>19.8</v>
+        <v>0</v>
       </c>
       <c r="H71" t="n">
-        <v>18.11</v>
+        <v>0</v>
       </c>
       <c r="I71" t="n">
-        <v>5.854</v>
+        <v>8.436999999999999</v>
       </c>
       <c r="J71" t="n">
-        <v>25.111</v>
+        <v>45.761</v>
       </c>
       <c r="K71" t="n">
-        <v>259</v>
+        <v>246.4</v>
       </c>
       <c r="L71" t="n">
-        <v>259</v>
+        <v>246.4</v>
       </c>
       <c r="M71" t="inlineStr">
         <is>
@@ -4701,36 +4689,36 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B72" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Customer_78</t>
+          <t>Customer_17</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>7323</v>
+        <v>9862</v>
       </c>
       <c r="E72" t="n">
-        <v>255.6</v>
+        <v>101.3</v>
       </c>
       <c r="F72" t="n">
-        <v>300.6</v>
+        <v>131.3</v>
       </c>
       <c r="G72" t="n">
-        <v>46.9</v>
+        <v>29.8</v>
       </c>
       <c r="H72" t="n">
-        <v>42.96</v>
+        <v>26.61</v>
       </c>
       <c r="I72" t="n">
-        <v>9.257</v>
+        <v>27.324</v>
       </c>
       <c r="J72" t="n">
-        <v>19.257</v>
+        <v>37.324</v>
       </c>
       <c r="K72" t="n">
         <v>282</v>
@@ -4744,24 +4732,24 @@
         </is>
       </c>
       <c r="N72" t="n">
-        <v>70.40000000000001</v>
+        <v>77</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B73" t="n">
         <v>1</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Customer_2</t>
+          <t>Customer_24</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -4770,10 +4758,10 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>6.2</v>
+        <v>18.6</v>
       </c>
       <c r="F73" t="n">
-        <v>36.2</v>
+        <v>48.6</v>
       </c>
       <c r="G73" t="n">
         <v>0</v>
@@ -4782,16 +4770,16 @@
         <v>0</v>
       </c>
       <c r="I73" t="n">
-        <v>32.335</v>
+        <v>25.462</v>
       </c>
       <c r="J73" t="n">
-        <v>42.335</v>
+        <v>49.555</v>
       </c>
       <c r="K73" t="n">
-        <v>273.8</v>
+        <v>255.5</v>
       </c>
       <c r="L73" t="n">
-        <v>273.8</v>
+        <v>255.5</v>
       </c>
       <c r="M73" t="inlineStr">
         <is>
@@ -4808,41 +4796,39 @@
         <v>19</v>
       </c>
       <c r="B74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Customer_24</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>VIR</t>
-        </is>
+          <t>Customer_10</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>6093</v>
       </c>
       <c r="E74" t="n">
-        <v>18.6</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F74" t="n">
-        <v>48.6</v>
+        <v>120.9</v>
       </c>
       <c r="G74" t="n">
-        <v>0</v>
+        <v>27.3</v>
       </c>
       <c r="H74" t="n">
-        <v>0</v>
+        <v>24.59</v>
       </c>
       <c r="I74" t="n">
-        <v>25.462</v>
+        <v>14.093</v>
       </c>
       <c r="J74" t="n">
-        <v>49.555</v>
+        <v>24.093</v>
       </c>
       <c r="K74" t="n">
-        <v>255.5</v>
+        <v>215.7</v>
       </c>
       <c r="L74" t="n">
-        <v>255.5</v>
+        <v>215.7</v>
       </c>
       <c r="M74" t="inlineStr">
         <is>
@@ -4856,42 +4842,44 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Customer_10</t>
-        </is>
-      </c>
-      <c r="D75" t="n">
-        <v>6093</v>
+          <t>Customer_28</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
       </c>
       <c r="E75" t="n">
-        <v>75.90000000000001</v>
+        <v>20.8</v>
       </c>
       <c r="F75" t="n">
-        <v>120.9</v>
+        <v>50.8</v>
       </c>
       <c r="G75" t="n">
-        <v>27.3</v>
+        <v>0</v>
       </c>
       <c r="H75" t="n">
-        <v>24.59</v>
+        <v>0</v>
       </c>
       <c r="I75" t="n">
-        <v>14.093</v>
+        <v>29.687</v>
       </c>
       <c r="J75" t="n">
-        <v>24.093</v>
+        <v>48.944</v>
       </c>
       <c r="K75" t="n">
-        <v>215.7</v>
+        <v>251.9</v>
       </c>
       <c r="L75" t="n">
-        <v>215.7</v>
+        <v>251.9</v>
       </c>
       <c r="M75" t="inlineStr">
         <is>
@@ -4908,51 +4896,53 @@
         <v>20</v>
       </c>
       <c r="B76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Customer_28</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>VIR</t>
-        </is>
+          <t>Customer_78</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>6599</v>
       </c>
       <c r="E76" t="n">
-        <v>20.8</v>
+        <v>90.2</v>
       </c>
       <c r="F76" t="n">
-        <v>50.8</v>
+        <v>135.2</v>
       </c>
       <c r="G76" t="n">
-        <v>0</v>
+        <v>39.4</v>
       </c>
       <c r="H76" t="n">
-        <v>0</v>
+        <v>36.09</v>
       </c>
       <c r="I76" t="n">
-        <v>29.687</v>
+        <v>9.257</v>
       </c>
       <c r="J76" t="n">
-        <v>39.687</v>
+        <v>19.257</v>
       </c>
       <c r="K76" t="n">
-        <v>255.5</v>
+        <v>282</v>
       </c>
       <c r="L76" t="n">
-        <v>255.5</v>
+        <v>282</v>
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N76" t="n">
-        <v>0</v>
-      </c>
-      <c r="O76" t="inlineStr"/>
+        <v>87.09999999999999</v>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -4987,13 +4977,13 @@
         <v>24.424</v>
       </c>
       <c r="J77" t="n">
-        <v>34.424</v>
+        <v>40.278</v>
       </c>
       <c r="K77" t="n">
-        <v>273</v>
+        <v>272.1</v>
       </c>
       <c r="L77" t="n">
-        <v>273</v>
+        <v>272.1</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
@@ -5007,44 +4997,42 @@
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Customer_38</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>VIR</t>
-        </is>
+          <t>Customer_36</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>7836</v>
       </c>
       <c r="E78" t="n">
-        <v>6.9</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="F78" t="n">
-        <v>51.9</v>
+        <v>131.1</v>
       </c>
       <c r="G78" t="n">
-        <v>0</v>
+        <v>33.5</v>
       </c>
       <c r="H78" t="n">
-        <v>0</v>
+        <v>30.69</v>
       </c>
       <c r="I78" t="n">
-        <v>32.721</v>
+        <v>5.854</v>
       </c>
       <c r="J78" t="n">
-        <v>42.721</v>
+        <v>15.854</v>
       </c>
       <c r="K78" t="n">
-        <v>272.8</v>
+        <v>229</v>
       </c>
       <c r="L78" t="n">
-        <v>272.8</v>
+        <v>229</v>
       </c>
       <c r="M78" t="inlineStr">
         <is>
@@ -5058,14 +5046,14 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B79" t="n">
         <v>1</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Customer_19</t>
+          <t>Customer_38</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -5074,10 +5062,10 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>19.8</v>
+        <v>6.9</v>
       </c>
       <c r="F79" t="n">
-        <v>64.8</v>
+        <v>51.9</v>
       </c>
       <c r="G79" t="n">
         <v>0</v>
@@ -5086,16 +5074,16 @@
         <v>0</v>
       </c>
       <c r="I79" t="n">
-        <v>16.088</v>
+        <v>32.721</v>
       </c>
       <c r="J79" t="n">
-        <v>26.088</v>
+        <v>42.721</v>
       </c>
       <c r="K79" t="n">
-        <v>261.6</v>
+        <v>272.8</v>
       </c>
       <c r="L79" t="n">
-        <v>261.6</v>
+        <v>272.8</v>
       </c>
       <c r="M79" t="inlineStr">
         <is>
@@ -5109,14 +5097,14 @@
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B80" t="n">
         <v>1</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Customer_17</t>
+          <t>Customer_19</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -5125,10 +5113,10 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>4.3</v>
+        <v>19.8</v>
       </c>
       <c r="F80" t="n">
-        <v>34.3</v>
+        <v>64.8</v>
       </c>
       <c r="G80" t="n">
         <v>0</v>
@@ -5137,16 +5125,16 @@
         <v>0</v>
       </c>
       <c r="I80" t="n">
-        <v>27.324</v>
+        <v>16.088</v>
       </c>
       <c r="J80" t="n">
-        <v>37.324</v>
+        <v>26.088</v>
       </c>
       <c r="K80" t="n">
-        <v>276.7</v>
+        <v>261.6</v>
       </c>
       <c r="L80" t="n">
-        <v>276.7</v>
+        <v>261.6</v>
       </c>
       <c r="M80" t="inlineStr">
         <is>
@@ -5160,7 +5148,7 @@
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B81" t="n">
         <v>1</v>
@@ -5220,7 +5208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5323,15 +5311,15 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>51.8</v>
+        <v>313.8</v>
       </c>
       <c r="D5" t="n">
         <v>282</v>
@@ -5340,7 +5328,7 @@
         <v>282</v>
       </c>
       <c r="F5" t="n">
-        <v>9.9</v>
+        <v>27.6</v>
       </c>
     </row>
     <row r="6">
@@ -5353,7 +5341,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>99.7</v>
+        <v>51.8</v>
       </c>
       <c r="D6" t="n">
         <v>282</v>
@@ -5362,7 +5350,7 @@
         <v>282</v>
       </c>
       <c r="F6" t="n">
-        <v>3.9</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="7">
@@ -5375,7 +5363,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>150.7</v>
+        <v>99.7</v>
       </c>
       <c r="D7" t="n">
         <v>282</v>
@@ -5384,20 +5372,20 @@
         <v>282</v>
       </c>
       <c r="F7" t="n">
-        <v>8.1</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>92.8</v>
+        <v>150.7</v>
       </c>
       <c r="D8" t="n">
         <v>282</v>
@@ -5406,7 +5394,7 @@
         <v>282</v>
       </c>
       <c r="F8" t="n">
-        <v>90.09999999999999</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="9">
@@ -5419,7 +5407,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>126.3</v>
+        <v>92.8</v>
       </c>
       <c r="D9" t="n">
         <v>282</v>
@@ -5428,7 +5416,7 @@
         <v>282</v>
       </c>
       <c r="F9" t="n">
-        <v>3.5</v>
+        <v>90.09999999999999</v>
       </c>
     </row>
     <row r="10">
@@ -5437,11 +5425,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>180.6</v>
+        <v>126.3</v>
       </c>
       <c r="D10" t="n">
         <v>282</v>
@@ -5450,7 +5438,7 @@
         <v>282</v>
       </c>
       <c r="F10" t="n">
-        <v>9.6</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="11">
@@ -5463,7 +5451,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>211.3</v>
+        <v>180.6</v>
       </c>
       <c r="D11" t="n">
         <v>282</v>
@@ -5472,12 +5460,12 @@
         <v>282</v>
       </c>
       <c r="F11" t="n">
-        <v>0.5</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -5485,7 +5473,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>100.4</v>
+        <v>211.3</v>
       </c>
       <c r="D12" t="n">
         <v>282</v>
@@ -5494,12 +5482,12 @@
         <v>282</v>
       </c>
       <c r="F12" t="n">
-        <v>80</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -5507,7 +5495,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>134.3</v>
+        <v>57.9</v>
       </c>
       <c r="D13" t="n">
         <v>282</v>
@@ -5516,20 +5504,20 @@
         <v>282</v>
       </c>
       <c r="F13" t="n">
-        <v>4.7</v>
+        <v>17.4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>192.4</v>
+        <v>91.7</v>
       </c>
       <c r="D14" t="n">
         <v>282</v>
@@ -5538,12 +5526,12 @@
         <v>282</v>
       </c>
       <c r="F14" t="n">
-        <v>11.7</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -5551,7 +5539,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>97.59999999999999</v>
+        <v>140.7</v>
       </c>
       <c r="D15" t="n">
         <v>282</v>
@@ -5560,20 +5548,20 @@
         <v>282</v>
       </c>
       <c r="F15" t="n">
-        <v>74.2</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>142.9</v>
+        <v>200.9</v>
       </c>
       <c r="D16" t="n">
         <v>282</v>
@@ -5582,20 +5570,20 @@
         <v>282</v>
       </c>
       <c r="F16" t="n">
-        <v>16.4</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>92.40000000000001</v>
+        <v>109.8</v>
       </c>
       <c r="D17" t="n">
         <v>282</v>
@@ -5604,20 +5592,20 @@
         <v>282</v>
       </c>
       <c r="F17" t="n">
-        <v>68.59999999999999</v>
+        <v>94.7</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>143.2</v>
+        <v>280.3</v>
       </c>
       <c r="D18" t="n">
         <v>282</v>
@@ -5626,20 +5614,20 @@
         <v>282</v>
       </c>
       <c r="F18" t="n">
-        <v>7.2</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>209.8</v>
+        <v>90.3</v>
       </c>
       <c r="D19" t="n">
         <v>282</v>
@@ -5648,20 +5636,20 @@
         <v>282</v>
       </c>
       <c r="F19" t="n">
-        <v>18.1</v>
+        <v>63.4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>270.2</v>
+        <v>188.4</v>
       </c>
       <c r="D20" t="n">
         <v>282</v>
@@ -5670,12 +5658,12 @@
         <v>282</v>
       </c>
       <c r="F20" t="n">
-        <v>24.9</v>
+        <v>36.1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -5683,7 +5671,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>73.59999999999999</v>
+        <v>297.5</v>
       </c>
       <c r="D21" t="n">
         <v>282</v>
@@ -5692,12 +5680,12 @@
         <v>282</v>
       </c>
       <c r="F21" t="n">
-        <v>41.9</v>
+        <v>41</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -5705,7 +5693,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>77.5</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="D22" t="n">
         <v>282</v>
@@ -5714,20 +5702,20 @@
         <v>282</v>
       </c>
       <c r="F22" t="n">
-        <v>67.59999999999999</v>
+        <v>41.9</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>140.3</v>
+        <v>77.5</v>
       </c>
       <c r="D23" t="n">
         <v>282</v>
@@ -5736,20 +5724,20 @@
         <v>282</v>
       </c>
       <c r="F23" t="n">
-        <v>16.2</v>
+        <v>67.59999999999999</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>65.8</v>
+        <v>140.3</v>
       </c>
       <c r="D24" t="n">
         <v>282</v>
@@ -5758,12 +5746,12 @@
         <v>282</v>
       </c>
       <c r="F24" t="n">
-        <v>30.3</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -5771,7 +5759,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>136.3</v>
+        <v>65.8</v>
       </c>
       <c r="D25" t="n">
         <v>282</v>
@@ -5780,12 +5768,12 @@
         <v>282</v>
       </c>
       <c r="F25" t="n">
-        <v>27.4</v>
+        <v>30.1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -5793,7 +5781,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>80.7</v>
+        <v>131.5</v>
       </c>
       <c r="D26" t="n">
         <v>282</v>
@@ -5802,12 +5790,12 @@
         <v>282</v>
       </c>
       <c r="F26" t="n">
-        <v>49.5</v>
+        <v>22.1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -5815,7 +5803,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>88.7</v>
+        <v>80.7</v>
       </c>
       <c r="D27" t="n">
         <v>282</v>
@@ -5824,20 +5812,20 @@
         <v>282</v>
       </c>
       <c r="F27" t="n">
-        <v>82.3</v>
+        <v>51.9</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>99</v>
+        <v>88.7</v>
       </c>
       <c r="D28" t="n">
         <v>282</v>
@@ -5846,29 +5834,95 @@
         <v>282</v>
       </c>
       <c r="F28" t="n">
-        <v>67.5</v>
+        <v>82.3</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
+        <v>16</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="D29" t="n">
+        <v>282</v>
+      </c>
+      <c r="E29" t="n">
+        <v>282</v>
+      </c>
+      <c r="F29" t="n">
+        <v>69.2</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
         <v>17</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="D30" t="n">
+        <v>282</v>
+      </c>
+      <c r="E30" t="n">
+        <v>282</v>
+      </c>
+      <c r="F30" t="n">
+        <v>42.1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>18</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>101.3</v>
+      </c>
+      <c r="D31" t="n">
+        <v>282</v>
+      </c>
+      <c r="E31" t="n">
+        <v>282</v>
+      </c>
+      <c r="F31" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>20</v>
+      </c>
+      <c r="B32" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="C29" t="n">
-        <v>255.6</v>
-      </c>
-      <c r="D29" t="n">
-        <v>282</v>
-      </c>
-      <c r="E29" t="n">
-        <v>282</v>
-      </c>
-      <c r="F29" t="n">
-        <v>70.40000000000001</v>
+      <c r="C32" t="n">
+        <v>90.2</v>
+      </c>
+      <c r="D32" t="n">
+        <v>282</v>
+      </c>
+      <c r="E32" t="n">
+        <v>282</v>
+      </c>
+      <c r="F32" t="n">
+        <v>87.09999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>